<commit_message>
Add parameterised what-if/scenario engine, config register and scenario workbook
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/Analytics_Question_Bank.xlsx
+++ b/data/Analytics_Question_Bank.xlsx
@@ -13,19 +13,21 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Q_Diagnostic" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Q_Predictive" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Q_Prescriptive" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Live_Answers" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_Commentary_Rules" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Commentary_Feed" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Refresh_Checklist" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Coverage_Map" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Q_WhatIf" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_Live_Answers" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Commentary_Rules" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Commentary_Feed" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Refresh_Checklist" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Coverage_Map" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'02_Q_Descriptive'!$A$4:$J$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'03_Q_Diagnostic'!$A$4:$J$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'04_Q_Predictive'!$A$4:$J$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'05_Q_Prescriptive'!$A$4:$J$26</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'06_Live_Answers'!$A$4:$I$48</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'08_Commentary_Feed'!$A$4:$J$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'06_Q_WhatIf'!$A$4:$J$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'07_Live_Answers'!$A$4:$I$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'09_Commentary_Feed'!$A$4:$J$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -152,7 +154,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -175,8 +177,11 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment/>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="3" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
@@ -186,12 +191,6 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -574,7 +573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -623,7 +622,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="70" customHeight="1">
+    <row r="8" ht="84" customHeight="1">
       <c r="B8" s="4" t="inlineStr">
         <is>
           <t>How it is organised</t>
@@ -631,7 +630,7 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>02–05: the questions, split into descriptive (what happened), diagnostic (why), predictive (what next) and prescriptive (what to do). 06: the live answer to every question that can be computed from the data, with a status flag. 07: the commentary rules (which causes to test, which actions to consider, when to act, who owns it). 08: the commentary actually triggered by the current data. 09: the refresh checklist and quality gates.</t>
+          <t>02–05: the questions, split into descriptive (what happened), diagnostic (why), predictive (what next) and prescriptive (what to do). 06: the what-if questions, answered by the scenario engine in VPT_WhatIf_Analysis.xlsx. 07: the live answer to every question that can be computed from the data, with a status flag. 08: the commentary rules (which causes to test, which actions to consider, when to act, who owns it). 09: the commentary actually triggered by the current data. 10: the refresh checklist and quality gates. 11: coverage against the BRD.</t>
         </is>
       </c>
     </row>
@@ -643,7 +642,7 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Every value in sheet 06 and every line in sheet 08 is computed from the current extract at build time and stamped with the data-as-at date. When the data is refreshed, re-run the refresh (script scripts/build_qa_workbook.py, or the equivalent scheduled job) and all answers, statuses and commentary lines are recomputed. Nothing is hard-coded.</t>
+          <t>Every value in sheet 07 and every line in sheet 09 is computed from the current extract at build time and stamped with the data-as-at date. When the data is refreshed, re-run the refresh (script scripts/build_qa_workbook.py, or the equivalent scheduled job) and all answers, statuses and commentary lines are recomputed. Nothing is hard-coded.</t>
         </is>
       </c>
     </row>
@@ -662,161 +661,173 @@
     <row r="11" ht="42" customHeight="1">
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Reading order at each refresh</t>
+          <t>Everything is configurable</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>1) Check sheet 09 quality gates are passed.  2) Read sheet 08 for what needs attention now.  3) Use sheet 06 to answer specific management questions.  4) Use 02–05 as the standing agenda for analysis.</t>
+          <t>All 15 thresholds and all 18 model assumptions live in config/parameters.json (parameter set v1.1). Changing a value there and re-running scripts/refresh_all.py changes every status flag, commentary line and scenario result — no code change, no retyping.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="42" customHeight="1">
       <c r="B12" s="4" t="inlineStr">
         <is>
+          <t>Reading order at each refresh</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>1) Check sheet 10 quality gates are passed.  2) Read sheet 09 for what needs attention now.  3) Use sheet 07 to answer specific management questions.  4) Use 02–06 as the standing agenda, including the what-if questions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="42" customHeight="1">
+      <c r="B13" s="4" t="inlineStr">
+        <is>
           <t>Cadence</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C13" s="5" t="inlineStr">
         <is>
           <t>Daily: data quality, stock-out risk on critical items.  Weekly: cover, expiry, commitments, procurement actions.  Monthly: consumption, ratio, budget, cost per beneficiary, commentary.  Quarterly: suppliers, price, efficiency, seasonality.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="28" customHeight="1">
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>Ownership</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>Business owner: Head of Procurement &amp; Supply Chain. Co-owners: Director Programme, Manager Finance &amp; Grants. Data owner: IT / BI. Each answered question carries a named owner in sheet 06.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="28" customHeight="1">
       <c r="B14" s="4" t="inlineStr">
         <is>
+          <t>Ownership</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Business owner: Head of Procurement &amp; Supply Chain. Co-owners: Director Programme, Manager Finance &amp; Grants. Data owner: IT / BI. Each answered question carries a named owner in sheet 06.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="28" customHeight="1">
+      <c r="B15" s="4" t="inlineStr">
+        <is>
           <t>Important note</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>Figures are computed from the current dataset extract. Organisation and supplier names are illustrative. Replace the extract with the Oracle feed before using this workbook in production.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="B16" s="6" t="inlineStr">
+    <row r="17">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>Headline position at this refresh</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="B17" s="7" t="inlineStr">
-        <is>
-          <t>Consumption value (excluding transfers)</t>
-        </is>
-      </c>
-      <c r="C17" s="8" t="inlineStr">
-        <is>
-          <t>PKR 261,575,946</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>Procurement investment</t>
+          <t>Consumption value (excluding transfers)</t>
         </is>
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>PKR 300,845,060</t>
+          <t>PKR 261,575,946</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Consumption-to-investment ratio</t>
+          <t>Procurement investment</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>0.87</t>
+          <t>PKR 300,845,060</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>Product budget / utilisation</t>
+          <t>Consumption-to-investment ratio</t>
         </is>
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>PKR 342,237,000  /  76%</t>
+          <t>0.87</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Unattributed consumption</t>
+          <t>Product budget / utilisation</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>PKR 6,271,241  (2.4%)</t>
+          <t>PKR 342,237,000  /  76%</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>Expired stock held</t>
+          <t>Unattributed consumption</t>
         </is>
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>PKR 783,764</t>
+          <t>PKR 6,271,241  (2.4%)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Open commitment</t>
+          <t>Expired stock held</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>PKR 4,467,951 across 320 open PO lines</t>
+          <t>PKR 783,764</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>Cost per beneficiary (period)</t>
+          <t>Open commitment</t>
         </is>
       </c>
       <c r="C24" s="8" t="inlineStr">
         <is>
-          <t>PKR 385</t>
+          <t>PKR 4,467,951 across 320 open PO lines</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="B25" s="7" t="inlineStr">
         <is>
+          <t>Cost per beneficiary (period)</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>PKR 385</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="7" t="inlineStr">
+        <is>
           <t>Question count</t>
         </is>
       </c>
-      <c r="C25" s="8" t="inlineStr">
+      <c r="C26" s="8" t="inlineStr">
         <is>
           <t>27 descriptive · 20 diagnostic · 16 predictive · 22 prescriptive</t>
         </is>
@@ -831,6 +842,838 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00E45756"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="58" customWidth="1" min="6" max="6"/>
+    <col width="46" customWidth="1" min="7" max="7"/>
+    <col width="52" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Live data commentary – what happened, why, so what, now what, when, who</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Generated from the data as at 2026-09-30. Each line is produced only because the metric breached its threshold in 01_Parameters; on refresh, lines move between Red, Amber and Green automatically.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>Ref</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>Current value</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>What happened (data)</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>Why it happened – causes to test</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>So what (impact)</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>What to do (action)</t>
+        </is>
+      </c>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>When to act</t>
+        </is>
+      </c>
+      <c r="J4" s="9" t="inlineStr">
+        <is>
+          <t>Owner / escalate</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="132" customHeight="1">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>CM-01</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>Consumption-to-investment ratio</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>0.87</t>
+        </is>
+      </c>
+      <c r="D5" s="18" t="inlineStr">
+        <is>
+          <t>Green</t>
+        </is>
+      </c>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>Consumption of PKR 261,575,946 against investment of PKR 300,845,060 gives a ratio of 0.87 for the period.</t>
+        </is>
+      </c>
+      <c r="F5" s="11" t="inlineStr">
+        <is>
+          <t>Ranked causes to test: (1) ordering ahead of need due to pack sizes or bulk discounts; (2) project start-up stock build; (3) slow issuing at service points; (4) drawdown of opening stock with no new purchase; (5) delayed receipts moving investment into a later period.</t>
+        </is>
+      </c>
+      <c r="G5" s="11" t="inlineStr">
+        <is>
+          <t>Value purchased but not yet used is cash tied up in store and at risk of expiry; a ratio far above 1.05 means consumption is being funded from stock and a stock-out will follow.</t>
+        </is>
+      </c>
+      <c r="H5" s="11" t="inlineStr">
+        <is>
+          <t>If below 0.80: defer the next purchase order, review pack-size-driven over-ordering, and check that issues are recorded daily. If above 1.05: confirm the stock position and re-base the requisition quantity.</t>
+        </is>
+      </c>
+      <c r="I5" s="11" t="inlineStr">
+        <is>
+          <t>At month close, before the next requisition cycle.</t>
+        </is>
+      </c>
+      <c r="J5" s="11" t="inlineStr">
+        <is>
+          <t>Head of Procurement → Director Finance &amp; Operations</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="132" customHeight="1">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>CM-02</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>Budget utilisation – Medical Consumables (FY2025-26)</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>151.4%</t>
+        </is>
+      </c>
+      <c r="D6" s="19" t="inlineStr">
+        <is>
+          <t>Red</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="inlineStr">
+        <is>
+          <t>Medical Consumables consumption of PKR 34,812,356 exceeds the approved budget of PKR 22,997,000 by PKR 11,815,356 (51.4%).</t>
+        </is>
+      </c>
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>Ranked causes to test: (1) price increase on a major item; (2) service volume higher than planned; (3) category budget under-estimated at planning; (4) mis-posting from another category; (5) wastage replacement purchases. Test price first, using the price-variance view (D-17).</t>
+        </is>
+      </c>
+      <c r="G6" s="11" t="inlineStr">
+        <is>
+          <t>An over-committed category can only be funded by taking budget from another line or by new money; left unresolved it becomes a donor-reporting exception in FY2025-26.</t>
+        </is>
+      </c>
+      <c r="H6" s="11" t="inlineStr">
+        <is>
+          <t>Record written commentary with the price/volume split; reallocate from an under-utilised category (see CM-03); tighten issue authorisation for the category; renegotiate the top two items by value.</t>
+        </is>
+      </c>
+      <c r="I6" s="11" t="inlineStr">
+        <is>
+          <t>Within 3 working days of the month close; reallocation before the fiscal year reaches 75% elapsed.</t>
+        </is>
+      </c>
+      <c r="J6" s="11" t="inlineStr">
+        <is>
+          <t>Manager Finance &amp; Grants → Director Finance &amp; Operations</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="132" customHeight="1">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>CM-03</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>Budget utilisation – Equipment (FY2026-27)</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>0.1%</t>
+        </is>
+      </c>
+      <c r="D7" s="19" t="inlineStr">
+        <is>
+          <t>Red</t>
+        </is>
+      </c>
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>Equipment budget of PKR 5,808,000 has used only PKR 6,782 (0.1%).</t>
+        </is>
+      </c>
+      <c r="F7" s="11" t="inlineStr">
+        <is>
+          <t>Ranked causes to test: (1) capital items stuck in approval or quotation; (2) requirement overstated at planning; (3) items recorded as consumables rather than equipment; (4) procurement deferred to the last quarter.</t>
+        </is>
+      </c>
+      <c r="G7" s="11" t="inlineStr">
+        <is>
+          <t>Under-utilisation is read by donors as slow implementation; at project end it becomes unspent budget and, if equipment is genuinely needed, a service-capability gap.</t>
+        </is>
+      </c>
+      <c r="H7" s="11" t="inlineStr">
+        <is>
+          <t>Review the equipment pipeline item by item; approve or cancel pending requests; either accelerate justified purchases or formally reallocate the budget to medicines and consumables before year end.</t>
+        </is>
+      </c>
+      <c r="I7" s="11" t="inlineStr">
+        <is>
+          <t>This quarter — capital purchases need the full procurement cycle before the fiscal year ends.</t>
+        </is>
+      </c>
+      <c r="J7" s="11" t="inlineStr">
+        <is>
+          <t>Head of Procurement → Director Programme</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="132" customHeight="1">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>CM-04</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>Unattributed consumption</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>2.4%</t>
+        </is>
+      </c>
+      <c r="D8" s="19" t="inlineStr">
+        <is>
+          <t>Red</t>
+        </is>
+      </c>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>PKR 6,271,241 of consumption (468 issue lines, 2.4% of value) is charged to a generic cost centre rather than a project. Worst month: Jan-2025.</t>
+        </is>
+      </c>
+      <c r="F8" s="11" t="inlineStr">
+        <is>
+          <t>Ranked causes to test: (1) a default or generic project code used as a shortcut at issue; (2) users not trained on project coding; (3) new project not yet set up in the system; (4) system default overriding the correct code. Cross-tabulate by user, warehouse and service point to identify the pattern.</t>
+        </is>
+      </c>
+      <c r="G8" s="11" t="inlineStr">
+        <is>
+          <t>Project-level consumption, cost per beneficiary and budget utilisation are all understated for the projects that actually consumed the stock, and overstated nowhere — the numbers do not add up to the total.</t>
+        </is>
+      </c>
+      <c r="H8" s="11" t="inlineStr">
+        <is>
+          <t>Correct retroactively where the consuming project is evidenced; make the project field mandatory and validated in Oracle; retrain the top users identified; add this exception to the monthly review agenda.</t>
+        </is>
+      </c>
+      <c r="I8" s="11" t="inlineStr">
+        <is>
+          <t>Correction within the current month; system control change within the quarter.</t>
+        </is>
+      </c>
+      <c r="J8" s="11" t="inlineStr">
+        <is>
+          <t>Head of Procurement (with IT) → Director Finance &amp; Operations</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="132" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>CM-05</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>Expired and near-expiry stock</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>PKR 783,764 expired; PKR 950,940 within 60 days</t>
+        </is>
+      </c>
+      <c r="D9" s="19" t="inlineStr">
+        <is>
+          <t>Red</t>
+        </is>
+      </c>
+      <c r="E9" s="11" t="inlineStr">
+        <is>
+          <t>PKR 783,764 of stock (1.9% of stock value) is already past expiry and not written off; a further PKR 950,940 expires within 60 days and PKR 636,720 within 90 days. Largest expired item: Hand Sanitiser 500 ml.</t>
+        </is>
+      </c>
+      <c r="F9" s="11" t="inlineStr">
+        <is>
+          <t>Ranked causes to test: (1) short-dated stock accepted at receipt or received as a donation; (2) over-ordering against an estimate rather than consumption; (3) stock held in the wrong warehouse or project; (4) protocol change making the item obsolete; (5) unrecorded consumption.</t>
+        </is>
+      </c>
+      <c r="G9" s="11" t="inlineStr">
+        <is>
+          <t>Direct, avoidable financial loss, plus a probable audit observation on stock management and donor reporting on commodity end-use.</t>
+        </is>
+      </c>
+      <c r="H9" s="11" t="inlineStr">
+        <is>
+          <t>Approve and record the write-off; redistribute the near-expiry balance to a project with demand; enforce first-expiry-first-out issue; reject short-dated deliveries at receipt; freeze ordering of the affected items.</t>
+        </is>
+      </c>
+      <c r="I9" s="11" t="inlineStr">
+        <is>
+          <t>Within 5 working days of the expiry flag; write-off before the financial year closes.</t>
+        </is>
+      </c>
+      <c r="J9" s="11" t="inlineStr">
+        <is>
+          <t>Stores in-charge → Head of Procurement</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="132" customHeight="1">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>CM-06</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>Stock cover / stock-out risk</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>3 items below 60 days; lowest 32 days (F-100 Therapeutic Milk 400 g)</t>
+        </is>
+      </c>
+      <c r="D10" s="20" t="inlineStr">
+        <is>
+          <t>Amber</t>
+        </is>
+      </c>
+      <c r="E10" s="11" t="inlineStr">
+        <is>
+          <t>0 items are below 30 days of cover and 3 below 60 days, against an average supplier lead time of 32 days.</t>
+        </is>
+      </c>
+      <c r="F10" s="11" t="inlineStr">
+        <is>
+          <t>Ranked causes to test: (1) lead time longer than the assumption used in planning; (2) demand surge above trend; (3) partial delivery or delayed GRN; (4) stock transferred out to another project; (5) pack size forcing under-supply.</t>
+        </is>
+      </c>
+      <c r="G10" s="11" t="inlineStr">
+        <is>
+          <t>A stock-out of a critical medicine interrupts service delivery and forces an emergency purchase at a higher price — the most expensive way to buy.</t>
+        </is>
+      </c>
+      <c r="H10" s="11" t="inlineStr">
+        <is>
+          <t>Raise a fast-track purchase for items where cover is below lead time; transfer stock from a warehouse with surplus cover; agree a temporary substitution with the clinical lead where clinically acceptable.</t>
+        </is>
+      </c>
+      <c r="I10" s="11" t="inlineStr">
+        <is>
+          <t>Immediately where cover is below lead time; same day for clinical items.</t>
+        </is>
+      </c>
+      <c r="J10" s="11" t="inlineStr">
+        <is>
+          <t>Stores in-charge (with Procurement) → Head of Procurement</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="132" customHeight="1">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>CM-07</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>Slow-moving and overstocked items</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>5 items, PKR 168,300; PKR 3,446,230 with over 180 days cover</t>
+        </is>
+      </c>
+      <c r="D11" s="20" t="inlineStr">
+        <is>
+          <t>Amber</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="inlineStr">
+        <is>
+          <t>5 items have no consumption in the last 90 days and PKR 3,446,230 of stock represents more than 180 days of cover. Stock on hand totals PKR 41,090,444.</t>
+        </is>
+      </c>
+      <c r="F11" s="11" t="inlineStr">
+        <is>
+          <t>Ranked causes to test: (1) demand over-estimated at requisition; (2) item superseded or removed from the protocol; (3) stock received for a project that has since reduced activity; (4) wrong warehouse allocation.</t>
+        </is>
+      </c>
+      <c r="G11" s="11" t="inlineStr">
+        <is>
+          <t>Blocked working capital and a future expiry loss; it also distorts the consumption-to-investment ratio.</t>
+        </is>
+      </c>
+      <c r="H11" s="11" t="inlineStr">
+        <is>
+          <t>Freeze re-ordering and set a review date; redistribute to a consuming project; correct the requirement formula with actual consumption; plan disposal or return for what cannot be consumed.</t>
+        </is>
+      </c>
+      <c r="I11" s="11" t="inlineStr">
+        <is>
+          <t>Freeze immediately; disposition before the expiry alert window.</t>
+        </is>
+      </c>
+      <c r="J11" s="11" t="inlineStr">
+        <is>
+          <t>Supply Chain Officer → Head of Procurement</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="132" customHeight="1">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>CM-08</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>Price variance</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>Average +16.2%; highest Diclofenac 75 mg Injection +19.4%</t>
+        </is>
+      </c>
+      <c r="D12" s="20" t="inlineStr">
+        <is>
+          <t>Amber</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="inlineStr">
+        <is>
+          <t>Across 77 items with comparable purchases, the weighted average unit price rose 16.2% between the first and latest purchase; Diclofenac 75 mg Injection rose from 28.99 to 34.63 (19.4%).</t>
+        </is>
+      </c>
+      <c r="F12" s="11" t="inlineStr">
+        <is>
+          <t>Ranked causes to test: (1) market or exchange-rate movement; (2) loss of contract price or supplier change; (3) specification or pack-size change; (4) emergency or split purchase at a higher price; (5) unit-of-measure error in the PO.</t>
+        </is>
+      </c>
+      <c r="G12" s="11" t="inlineStr">
+        <is>
+          <t>Price movement consumes budget without any change in service volume, so activity has to be reduced later in the year unless it is negotiated or re-budgeted.</t>
+        </is>
+      </c>
+      <c r="H12" s="11" t="inlineStr">
+        <is>
+          <t>Re-quote or invoke contract terms for the top five risers; consolidate demand to restore volume discounts; verify specification and UOM; record the price effect separately in the variance commentary.</t>
+        </is>
+      </c>
+      <c r="I12" s="11" t="inlineStr">
+        <is>
+          <t>Before the next contract or purchase cycle.</t>
+        </is>
+      </c>
+      <c r="J12" s="11" t="inlineStr">
+        <is>
+          <t>Procurement Officer → Head of Procurement</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="132" customHeight="1">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>CM-09</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>Open commitments and cancelled orders</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>PKR 4,467,951 open; 847 lines cancelled (PKR 18,943,642)</t>
+        </is>
+      </c>
+      <c r="D13" s="20" t="inlineStr">
+        <is>
+          <t>Amber</t>
+        </is>
+      </c>
+      <c r="E13" s="11" t="inlineStr">
+        <is>
+          <t>320 PO lines worth PKR 4,467,951 remain un-received, and 847 lines worth PKR 18,943,642 were cancelled in the period.</t>
+        </is>
+      </c>
+      <c r="F13" s="11" t="inlineStr">
+        <is>
+          <t>Ranked causes to test: (1) supplier capacity or import delay; (2) budget hold or approval delay; (3) requirement changed after ordering; (4) split ordering to stay within approval limits.</t>
+        </is>
+      </c>
+      <c r="G13" s="11" t="inlineStr">
+        <is>
+          <t>Open commitments are future cash outflows and future stock; cancellations indicate that requisitions were raised before the need was firm, which wastes procurement capacity.</t>
+        </is>
+      </c>
+      <c r="H13" s="11" t="inlineStr">
+        <is>
+          <t>Confirm delivery dates in writing; re-plan or cancel the balance where the need has changed; review approval thresholds if split ordering is evident; use the commitment figure in cash planning.</t>
+        </is>
+      </c>
+      <c r="I13" s="11" t="inlineStr">
+        <is>
+          <t>Weekly review; escalate any line open for more than 30 days.</t>
+        </is>
+      </c>
+      <c r="J13" s="11" t="inlineStr">
+        <is>
+          <t>Procurement Officer → Manager Finance</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="132" customHeight="1">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>CM-10</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>Projects ending soon with unspent budget</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>6 projects; PKR 136,478,187 unspent</t>
+        </is>
+      </c>
+      <c r="D14" s="19" t="inlineStr">
+        <is>
+          <t>Red</t>
+        </is>
+      </c>
+      <c r="E14" s="11" t="inlineStr">
+        <is>
+          <t>6 projects end within 120 days with a combined PKR 136,478,187 of budget unspent (largest: Maternal &amp; Child Health Programme - Kora, PKR 33,322,723).</t>
+        </is>
+      </c>
+      <c r="F14" s="11" t="inlineStr">
+        <is>
+          <t>Ranked causes to test: (1) activity slower than plan; (2) budget allocated but never requisitioned; (3) consumption recorded against another project; (4) procurement capacity constraint; (5) budget overstated at award.</t>
+        </is>
+      </c>
+      <c r="G14" s="11" t="inlineStr">
+        <is>
+          <t>Unspent budget at project end is reported to donors as under-delivery and may be recovered; correcting it at the last minute usually produces poor-quality spending.</t>
+        </is>
+      </c>
+      <c r="H14" s="11" t="inlineStr">
+        <is>
+          <t>Prepare an end-of-project plan now: accelerate committed activity, procure only justified items, request a no-cost extension where activity remains, or return the balance formally.</t>
+        </is>
+      </c>
+      <c r="I14" s="11" t="inlineStr">
+        <is>
+          <t>This month — the procurement cycle must still fit inside the remaining period.</t>
+        </is>
+      </c>
+      <c r="J14" s="11" t="inlineStr">
+        <is>
+          <t>Programme Manager (with Finance) → Director Programme</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="132" customHeight="1">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>CM-11</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>Projected FY2026-27 funding position</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>projected PKR 67,536,754 vs budget PKR 67,078,000; gap PKR 458,754</t>
+        </is>
+      </c>
+      <c r="D15" s="19" t="inlineStr">
+        <is>
+          <t>Red</t>
+        </is>
+      </c>
+      <c r="E15" s="11" t="inlineStr">
+        <is>
+          <t>With 3 months elapsed and PKR 33,768,377 consumed, the burn rate of PKR 11,256,126 per month projects PKR 67,536,754 for the full year against a product budget of PKR 67,078,000.</t>
+        </is>
+      </c>
+      <c r="F15" s="11" t="inlineStr">
+        <is>
+          <t>Ranked causes to test: (1) budget phasing not yet loaded for the year; (2) genuine under-budgeting against price inflation; (3) consumption running above the planned service volume; (4) prior-year carry-over spend landing in this year.</t>
+        </is>
+      </c>
+      <c r="G15" s="11" t="inlineStr">
+        <is>
+          <t>If the gap is real, service levels cannot be maintained for the full year and the shortfall appears unannounced in the last quarter.</t>
+        </is>
+      </c>
+      <c r="H15" s="11" t="inlineStr">
+        <is>
+          <t>Confirm budget phasing with Finance first; if the gap is real, quantify it by project and category, prioritise spending on critical items, and raise a funding request or reprioritise activity with the donor.</t>
+        </is>
+      </c>
+      <c r="I15" s="11" t="inlineStr">
+        <is>
+          <t>Now, at the first quarter of the fiscal year — not at the ninth month.</t>
+        </is>
+      </c>
+      <c r="J15" s="11" t="inlineStr">
+        <is>
+          <t>Manager Finance &amp; Grants → Director Finance &amp; Operations</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="132" customHeight="1">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>CM-12</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>Cost per beneficiary (peer comparison)</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>overall PKR 385; range Hepatitis B &amp; C Screening -  PKR 227 to Nutrition Stabilisation Cent PKR 500</t>
+        </is>
+      </c>
+      <c r="D16" s="20" t="inlineStr">
+        <is>
+          <t>Amber</t>
+        </is>
+      </c>
+      <c r="E16" s="11" t="inlineStr">
+        <is>
+          <t>Product cost per beneficiary is PKR 385 across the portfolio, but ranges from PKR 227 in Hepatitis B &amp; C Screening - Keamari to PKR 500 in Nutrition Stabilisation Centre - Malir (a spread of 120.8%).</t>
+        </is>
+      </c>
+      <c r="F16" s="11" t="inlineStr">
+        <is>
+          <t>Ranked causes to test: (1) case mix and acuity of the service; (2) price paid and supplier terms; (3) service volume below facility capacity; (4) wastage and expiry inflating cost; (5) one-off stock build in the period.</t>
+        </is>
+      </c>
+      <c r="G16" s="11" t="inlineStr">
+        <is>
+          <t>A high cost per beneficiary relative to peers is the first question a donor asks; without an explanation it is read as inefficiency.</t>
+        </is>
+      </c>
+      <c r="H16" s="11" t="inlineStr">
+        <is>
+          <t>Normalise for category mix before drawing conclusions; address the identified driver (price, volume or waste); set an efficiency target for the next quarter and report the measure with its methodology.</t>
+        </is>
+      </c>
+      <c r="I16" s="11" t="inlineStr">
+        <is>
+          <t>Quarterly review, with the methodology published alongside the first report.</t>
+        </is>
+      </c>
+      <c r="J16" s="11" t="inlineStr">
+        <is>
+          <t>Director Programme → Executive management</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="132" customHeight="1">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>CM-13</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>Seasonality and peak readiness</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>peak month Aug-2025 (PKR 14,731,533); seasonal index highest in Jan at 1.23</t>
+        </is>
+      </c>
+      <c r="D17" s="20" t="inlineStr">
+        <is>
+          <t>Amber</t>
+        </is>
+      </c>
+      <c r="E17" s="11" t="inlineStr">
+        <is>
+          <t>Consumption peaks in Aug-2025 at PKR 14,731,533, 52.1% above the period average; the seasonal index is highest in Jan (1.23×) and lowest in Mar (0.83×).</t>
+        </is>
+      </c>
+      <c r="F17" s="11" t="inlineStr">
+        <is>
+          <t>Seasonal demand is driven by disease pattern (diarrhoeal and vector-borne illness in the monsoon months), campaign activity and beneficiary inflow; the peak is structural, not a one-off.</t>
+        </is>
+      </c>
+      <c r="G17" s="11" t="inlineStr">
+        <is>
+          <t>If stock is purchased during the surge rather than before it, the peak is met with emergency purchases at higher prices and with stock-outs at the moment of greatest need.</t>
+        </is>
+      </c>
+      <c r="H17" s="11" t="inlineStr">
+        <is>
+          <t>Pre-position peak quantities at least one lead time before the peak month; align the purchase plan and warehouse capacity with the seasonal index; review the index each quarter.</t>
+        </is>
+      </c>
+      <c r="I17" s="11" t="inlineStr">
+        <is>
+          <t>Two months before the peak season, every year.</t>
+        </is>
+      </c>
+      <c r="J17" s="11" t="inlineStr">
+        <is>
+          <t>Supply Chain Officer → Head of Procurement</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="132" customHeight="1">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>CM-14</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>Data quality and load integrity</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>8 duplicate receipts; 59 zero-price lines; 2 inactive items; 1 blacklisted supplier</t>
+        </is>
+      </c>
+      <c r="D18" s="20" t="inlineStr">
+        <is>
+          <t>Amber</t>
+        </is>
+      </c>
+      <c r="E18" s="11" t="inlineStr">
+        <is>
+          <t>The load contains 8 duplicate receipt candidates, 59 purchase lines at zero value, 2 inactive items with transaction history and 1 blacklisted supplier still appearing in purchase orders.</t>
+        </is>
+      </c>
+      <c r="F18" s="11" t="inlineStr">
+        <is>
+          <t>Ranked causes to test: (1) double posting in the source system; (2) in-kind or donated stock genuinely at zero value; (3) master data not maintained after item or supplier deactivation; (4) extract mapping or UOM error.</t>
+        </is>
+      </c>
+      <c r="G18" s="11" t="inlineStr">
+        <is>
+          <t>Each defect flows into a reported KPI: duplicates inflate stock and receipts, zero prices distort average price, and inactive data hides real consumption.</t>
+        </is>
+      </c>
+      <c r="H18" s="11" t="inlineStr">
+        <is>
+          <t>Deduplicate and correct at source before the next refresh; exclude zero-value lines from price analysis and disclose them as in-kind; clean the master data; add the check to the load gate.</t>
+        </is>
+      </c>
+      <c r="I18" s="11" t="inlineStr">
+        <is>
+          <t>Before the next refresh; defects recurring for three periods require a process change.</t>
+        </is>
+      </c>
+      <c r="J18" s="11" t="inlineStr">
+        <is>
+          <t>IT / BI → Head of Procurement</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Rule: no commentary without a number, no number without a cause, no cause without an action, no action without an owner and a date.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:J18"/>
+  <mergeCells count="1">
+    <mergeCell ref="A2:J2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="0072B7B2"/>
@@ -1166,14 +2009,14 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="004C78A8"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1310,7 +2153,7 @@
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>05 + 09</t>
+          <t>05 + 10</t>
         </is>
       </c>
       <c r="D8" s="10" t="inlineStr">
@@ -1324,43 +2167,68 @@
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
-          <t>Total questions: 85</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>What-if</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>06 + VPT_WhatIf_Analysis.xlsx</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>Quantify the effect of a driver moving, and choose a response</t>
+        </is>
+      </c>
+      <c r="E9" s="11" t="inlineStr">
+        <is>
+          <t>FR-49 to FR-53, §14.4 parameterisation</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Total questions: 99</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>Refresh-driven design</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="22" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="21" t="inlineStr">
         <is>
           <t>•  The question text, purpose, data fields, logic and owner are stable — they are the standing analysis agenda.</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="22" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="21" t="inlineStr">
         <is>
           <t>•  The answer, the status flag and the commentary text are recomputed from the data at each refresh and stamped with the as-at date.</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="22" t="inlineStr">
-        <is>
-          <t>•  Thresholds live in 01_Parameters so that a change of tolerance changes every status and commentary line consistently.</t>
-        </is>
-      </c>
-    </row>
     <row r="16">
-      <c r="A16" s="22" t="inlineStr">
+      <c r="A16" s="21" t="inlineStr">
+        <is>
+          <t>•  Thresholds and model assumptions live in config/parameters.json and are displayed in 01_Parameters, so a change of tolerance or assumption changes every status, commentary line and scenario consistently.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="21" t="inlineStr">
         <is>
           <t>•  Where a question cannot yet be answered (for example a missing programme data field), it stays in the bank with a data-gap note rather than being removed.</t>
         </is>
@@ -1381,7 +2249,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:G44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1445,17 +2313,17 @@
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
-          <t>auto</t>
+          <t>auto (from load log)</t>
         </is>
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>Later of last successful load and last closed period</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="E5" s="11" t="inlineStr">
         <is>
-          <t>Shown on every page; drives all 'as at' labels</t>
+          <t>Later of last successful load and last closed period; shown on every page and stamped on every answer</t>
         </is>
       </c>
     </row>
@@ -1467,12 +2335,12 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>Consumption-to-investment ratio – acceptable band</t>
+          <t>Consumption-to-investment ratio band</t>
         </is>
       </c>
       <c r="C6" s="10" t="inlineStr">
         <is>
-          <t>0.80 – 1.05</t>
+          <t>0.80-1.05</t>
         </is>
       </c>
       <c r="D6" s="10" t="inlineStr">
@@ -1494,7 +2362,7 @@
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>Consumption variance vs budget – investigate above</t>
+          <t>Consumption variance vs budget - investigate above</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
@@ -1509,7 +2377,7 @@
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>Variance beyond this band requires written commentary</t>
+          <t>Beyond this band the variance requires written commentary and an owner</t>
         </is>
       </c>
     </row>
@@ -1526,17 +2394,17 @@
       </c>
       <c r="C8" s="10" t="inlineStr">
         <is>
-          <t>PKR 250,000 or 10% of category budget</t>
+          <t>PKR 250,000</t>
         </is>
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>PKR / %</t>
+          <t>PKR</t>
         </is>
       </c>
       <c r="E8" s="11" t="inlineStr">
         <is>
-          <t>Whichever is lower; below this, comment at category level only</t>
+          <t>PKR 250,000 or 10% of the category budget, whichever is lower</t>
         </is>
       </c>
     </row>
@@ -1548,12 +2416,12 @@
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>Days of cover – critical threshold</t>
+          <t>Days of cover - critical threshold</t>
         </is>
       </c>
       <c r="C9" s="10" t="inlineStr">
         <is>
-          <t>&lt; 30 days</t>
+          <t>30</t>
         </is>
       </c>
       <c r="D9" s="10" t="inlineStr">
@@ -1563,7 +2431,7 @@
       </c>
       <c r="E9" s="11" t="inlineStr">
         <is>
-          <t>Raise purchase requisition immediately</t>
+          <t>Raise a purchase requisition or transfer immediately</t>
         </is>
       </c>
     </row>
@@ -1575,12 +2443,12 @@
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>Days of cover – watch threshold</t>
+          <t>Days of cover - watch threshold</t>
         </is>
       </c>
       <c r="C10" s="10" t="inlineStr">
         <is>
-          <t>30 – 60 days</t>
+          <t>60</t>
         </is>
       </c>
       <c r="D10" s="10" t="inlineStr">
@@ -1590,7 +2458,7 @@
       </c>
       <c r="E10" s="11" t="inlineStr">
         <is>
-          <t>Include in next monthly purchase plan</t>
+          <t>Include in the next monthly purchase plan</t>
         </is>
       </c>
     </row>
@@ -1602,12 +2470,12 @@
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>Days of cover – overstock threshold</t>
+          <t>Days of cover - overstock threshold</t>
         </is>
       </c>
       <c r="C11" s="10" t="inlineStr">
         <is>
-          <t>&gt; 180 days</t>
+          <t>180</t>
         </is>
       </c>
       <c r="D11" s="10" t="inlineStr">
@@ -1617,7 +2485,7 @@
       </c>
       <c r="E11" s="11" t="inlineStr">
         <is>
-          <t>Freeze re-ordering; review allocation to other projects</t>
+          <t>Freeze re-ordering and review redistribution</t>
         </is>
       </c>
     </row>
@@ -1634,7 +2502,7 @@
       </c>
       <c r="C12" s="10" t="inlineStr">
         <is>
-          <t>60 / 90 / 180 days</t>
+          <t>60</t>
         </is>
       </c>
       <c r="D12" s="10" t="inlineStr">
@@ -1656,7 +2524,7 @@
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>Price variance – investigate above</t>
+          <t>Price variance - investigate above</t>
         </is>
       </c>
       <c r="C13" s="10" t="inlineStr">
@@ -1671,7 +2539,7 @@
       </c>
       <c r="E13" s="11" t="inlineStr">
         <is>
-          <t>Compare supplier quotes; check contract validity</t>
+          <t>Compare supplier quotes and check contract validity</t>
         </is>
       </c>
     </row>
@@ -1688,7 +2556,7 @@
       </c>
       <c r="C14" s="10" t="inlineStr">
         <is>
-          <t>1.0% of value</t>
+          <t>1%</t>
         </is>
       </c>
       <c r="D14" s="10" t="inlineStr">
@@ -1698,7 +2566,7 @@
       </c>
       <c r="E14" s="11" t="inlineStr">
         <is>
-          <t>Above this, escalate to project coding owner</t>
+          <t>Above this, escalate to the project-coding owner</t>
         </is>
       </c>
     </row>
@@ -1715,7 +2583,7 @@
       </c>
       <c r="C15" s="10" t="inlineStr">
         <is>
-          <t>30 days</t>
+          <t>30</t>
         </is>
       </c>
       <c r="D15" s="10" t="inlineStr">
@@ -1725,7 +2593,7 @@
       </c>
       <c r="E15" s="11" t="inlineStr">
         <is>
-          <t>Escalate to Head of Procurement</t>
+          <t>Escalate to the Head of Procurement</t>
         </is>
       </c>
     </row>
@@ -1742,7 +2610,7 @@
       </c>
       <c r="C16" s="10" t="inlineStr">
         <is>
-          <t>6 and 12 months</t>
+          <t>6</t>
         </is>
       </c>
       <c r="D16" s="10" t="inlineStr">
@@ -1752,7 +2620,7 @@
       </c>
       <c r="E16" s="11" t="inlineStr">
         <is>
-          <t>Zero issues in lookback with stock on hand = slow-moving</t>
+          <t>Zero issues in the lookback with stock on hand = slow-moving</t>
         </is>
       </c>
     </row>
@@ -1769,7 +2637,7 @@
       </c>
       <c r="C17" s="10" t="inlineStr">
         <is>
-          <t>90 days plus supplier lead time</t>
+          <t>90</t>
         </is>
       </c>
       <c r="D17" s="10" t="inlineStr">
@@ -1796,17 +2664,17 @@
       </c>
       <c r="C18" s="10" t="inlineStr">
         <is>
-          <t>0 critical items with &lt; 15 days cover</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D18" s="10" t="inlineStr">
         <is>
-          <t>Count</t>
+          <t>Items</t>
         </is>
       </c>
       <c r="E18" s="11" t="inlineStr">
         <is>
-          <t>Any breach is a service risk</t>
+          <t>Any critical item below 15 days of cover is a service risk</t>
         </is>
       </c>
     </row>
@@ -1823,7 +2691,7 @@
       </c>
       <c r="C19" s="10" t="inlineStr">
         <is>
-          <t>in line with elapsed project time ± 15%</t>
+          <t>elapsed+/-15%</t>
         </is>
       </c>
       <c r="D19" s="10" t="inlineStr">
@@ -1833,14 +2701,695 @@
       </c>
       <c r="E19" s="11" t="inlineStr">
         <is>
-          <t>Under or over this band needs explanation</t>
+          <t>Under or over this band requires explanation</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="12" t="inlineStr">
-        <is>
-          <t>Threshold values are defaults proposed in the BRD. Approval: Head of Procurement; changes recorded in the change log.</t>
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Parameter set v1.1 — these values are loaded from config/parameters.json, not typed here. Approval: Head of Procurement; every change is recorded with the old value, the new value, the reason and the effective date, and applies from the next refresh.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>Model parameters that drive the what-if engine (see VPT_WhatIf_Analysis.xlsx)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="32" customHeight="1">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>Key</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="inlineStr">
+        <is>
+          <t>Parameter</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="E24" s="9" t="inlineStr">
+        <is>
+          <t>Range</t>
+        </is>
+      </c>
+      <c r="F24" s="9" t="inlineStr">
+        <is>
+          <t>Basis</t>
+        </is>
+      </c>
+      <c r="G24" s="9" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="10" t="inlineStr">
+        <is>
+          <t>demand_growth_pct</t>
+        </is>
+      </c>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>Demand growth (annual)</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="D25" s="10" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E25" s="10" t="inlineStr">
+        <is>
+          <t>-0.3 – 0.5</t>
+        </is>
+      </c>
+      <c r="F25" s="11" t="inlineStr">
+        <is>
+          <t>Programme growth trend over the reporting window</t>
+        </is>
+      </c>
+      <c r="G25" s="10" t="inlineStr">
+        <is>
+          <t>Programme</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>service_volume_growth_pct</t>
+        </is>
+      </c>
+      <c r="B26" s="11" t="inlineStr">
+        <is>
+          <t>Service volume (beneficiary) growth</t>
+        </is>
+      </c>
+      <c r="C26" s="12" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="D26" s="10" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E26" s="10" t="inlineStr">
+        <is>
+          <t>-0.3 – 0.5</t>
+        </is>
+      </c>
+      <c r="F26" s="11" t="inlineStr">
+        <is>
+          <t>Beneficiary trend in the service-delivery data</t>
+        </is>
+      </c>
+      <c r="G26" s="10" t="inlineStr">
+        <is>
+          <t>Programme</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>activity_factor</t>
+        </is>
+      </c>
+      <c r="B27" s="11" t="inlineStr">
+        <is>
+          <t>Project activity factor (next 12 months)</t>
+        </is>
+      </c>
+      <c r="C27" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" s="10" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="E27" s="10" t="inlineStr">
+        <is>
+          <t>0.1 – 1.0</t>
+        </is>
+      </c>
+      <c r="F27" s="11" t="inlineStr">
+        <is>
+          <t>Share of the next 12 months in which at least one project is active (from project end dates)</t>
+        </is>
+      </c>
+      <c r="G27" s="10" t="inlineStr">
+        <is>
+          <t>Programme</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>price_inflation_pct</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>Price inflation (annual)</t>
+        </is>
+      </c>
+      <c r="C28" s="12" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="D28" s="10" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E28" s="10" t="inlineStr">
+        <is>
+          <t>-0.1 – 0.4</t>
+        </is>
+      </c>
+      <c r="F28" s="11" t="inlineStr">
+        <is>
+          <t>Weighted average unit-price movement in the purchase history</t>
+        </is>
+      </c>
+      <c r="G28" s="10" t="inlineStr">
+        <is>
+          <t>Procurement</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="10" t="inlineStr">
+        <is>
+          <t>price_shock_pct</t>
+        </is>
+      </c>
+      <c r="B29" s="11" t="inlineStr">
+        <is>
+          <t>One-off price shock</t>
+        </is>
+      </c>
+      <c r="C29" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="10" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E29" s="10" t="inlineStr">
+        <is>
+          <t>-0.2 – 0.5</t>
+        </is>
+      </c>
+      <c r="F29" s="11" t="inlineStr">
+        <is>
+          <t>Scenario lever for a market, currency or contract event</t>
+        </is>
+      </c>
+      <c r="G29" s="10" t="inlineStr">
+        <is>
+          <t>Procurement</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="10" t="inlineStr">
+        <is>
+          <t>bulk_discount_pct</t>
+        </is>
+      </c>
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>Bulk / framework discount</t>
+        </is>
+      </c>
+      <c r="C30" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" s="10" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E30" s="10" t="inlineStr">
+        <is>
+          <t>0.0 – 0.25</t>
+        </is>
+      </c>
+      <c r="F30" s="11" t="inlineStr">
+        <is>
+          <t>Negotiated discount on consolidated demand</t>
+        </is>
+      </c>
+      <c r="G30" s="10" t="inlineStr">
+        <is>
+          <t>Procurement</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="10" t="inlineStr">
+        <is>
+          <t>lead_time_multiplier</t>
+        </is>
+      </c>
+      <c r="B31" s="11" t="inlineStr">
+        <is>
+          <t>Supplier lead-time multiplier</t>
+        </is>
+      </c>
+      <c r="C31" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" s="10" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="E31" s="10" t="inlineStr">
+        <is>
+          <t>0.5 – 3.0</t>
+        </is>
+      </c>
+      <c r="F31" s="11" t="inlineStr">
+        <is>
+          <t>1.00 = current average lead time of the supplier base</t>
+        </is>
+      </c>
+      <c r="G31" s="10" t="inlineStr">
+        <is>
+          <t>Procurement</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="10" t="inlineStr">
+        <is>
+          <t>supplier_reliability_pct</t>
+        </is>
+      </c>
+      <c r="B32" s="11" t="inlineStr">
+        <is>
+          <t>Supplier on-time reliability</t>
+        </is>
+      </c>
+      <c r="C32" s="12" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="D32" s="10" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E32" s="10" t="inlineStr">
+        <is>
+          <t>0.4 – 1.0</t>
+        </is>
+      </c>
+      <c r="F32" s="11" t="inlineStr">
+        <is>
+          <t>Share of orders received within the agreed lead time</t>
+        </is>
+      </c>
+      <c r="G32" s="10" t="inlineStr">
+        <is>
+          <t>Procurement</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="10" t="inlineStr">
+        <is>
+          <t>target_cover_days</t>
+        </is>
+      </c>
+      <c r="B33" s="11" t="inlineStr">
+        <is>
+          <t>Target stock cover</t>
+        </is>
+      </c>
+      <c r="C33" s="10" t="n">
+        <v>90</v>
+      </c>
+      <c r="D33" s="10" t="inlineStr">
+        <is>
+          <t>Days</t>
+        </is>
+      </c>
+      <c r="E33" s="10" t="inlineStr">
+        <is>
+          <t>15 – 240</t>
+        </is>
+      </c>
+      <c r="F33" s="11" t="inlineStr">
+        <is>
+          <t>Policy: cover to hold after each purchase cycle</t>
+        </is>
+      </c>
+      <c r="G33" s="10" t="inlineStr">
+        <is>
+          <t>Head of Procurement</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="10" t="inlineStr">
+        <is>
+          <t>safety_stock_days</t>
+        </is>
+      </c>
+      <c r="B34" s="11" t="inlineStr">
+        <is>
+          <t>Safety stock</t>
+        </is>
+      </c>
+      <c r="C34" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="D34" s="10" t="inlineStr">
+        <is>
+          <t>Days</t>
+        </is>
+      </c>
+      <c r="E34" s="10" t="inlineStr">
+        <is>
+          <t>0 – 90</t>
+        </is>
+      </c>
+      <c r="F34" s="11" t="inlineStr">
+        <is>
+          <t>Buffer against lead-time and demand variability</t>
+        </is>
+      </c>
+      <c r="G34" s="10" t="inlineStr">
+        <is>
+          <t>Head of Procurement</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="10" t="inlineStr">
+        <is>
+          <t>max_cover_days</t>
+        </is>
+      </c>
+      <c r="B35" s="11" t="inlineStr">
+        <is>
+          <t>Maximum acceptable cover</t>
+        </is>
+      </c>
+      <c r="C35" s="10" t="n">
+        <v>180</v>
+      </c>
+      <c r="D35" s="10" t="inlineStr">
+        <is>
+          <t>Days</t>
+        </is>
+      </c>
+      <c r="E35" s="10" t="inlineStr">
+        <is>
+          <t>60 – 365</t>
+        </is>
+      </c>
+      <c r="F35" s="11" t="inlineStr">
+        <is>
+          <t>Above this, stock counts as overstocked</t>
+        </is>
+      </c>
+      <c r="G35" s="10" t="inlineStr">
+        <is>
+          <t>Supply chain</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="10" t="inlineStr">
+        <is>
+          <t>expiry_alert_days</t>
+        </is>
+      </c>
+      <c r="B36" s="11" t="inlineStr">
+        <is>
+          <t>Expiry alert window</t>
+        </is>
+      </c>
+      <c r="C36" s="10" t="n">
+        <v>60</v>
+      </c>
+      <c r="D36" s="10" t="inlineStr">
+        <is>
+          <t>Days</t>
+        </is>
+      </c>
+      <c r="E36" s="10" t="inlineStr">
+        <is>
+          <t>15 – 180</t>
+        </is>
+      </c>
+      <c r="F36" s="11" t="inlineStr">
+        <is>
+          <t>Alert before expiry for redistribution or consumption</t>
+        </is>
+      </c>
+      <c r="G36" s="10" t="inlineStr">
+        <is>
+          <t>Stores</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="10" t="inlineStr">
+        <is>
+          <t>wastage_rate_pct</t>
+        </is>
+      </c>
+      <c r="B37" s="11" t="inlineStr">
+        <is>
+          <t>Wastage / write-off rate</t>
+        </is>
+      </c>
+      <c r="C37" s="12" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="D37" s="10" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E37" s="10" t="inlineStr">
+        <is>
+          <t>0.0 – 0.1</t>
+        </is>
+      </c>
+      <c r="F37" s="11" t="inlineStr">
+        <is>
+          <t>Observed expired and damaged stock as a share of consumption</t>
+        </is>
+      </c>
+      <c r="G37" s="10" t="inlineStr">
+        <is>
+          <t>Stores</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="10" t="inlineStr">
+        <is>
+          <t>redistribution_share_pct</t>
+        </is>
+      </c>
+      <c r="B38" s="11" t="inlineStr">
+        <is>
+          <t>Overstock redistributed</t>
+        </is>
+      </c>
+      <c r="C38" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D38" s="10" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E38" s="10" t="inlineStr">
+        <is>
+          <t>0.0 – 1.0</t>
+        </is>
+      </c>
+      <c r="F38" s="11" t="inlineStr">
+        <is>
+          <t>Share of excess stock moved to a project with demand instead of being written off</t>
+        </is>
+      </c>
+      <c r="G38" s="10" t="inlineStr">
+        <is>
+          <t>Supply chain</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="10" t="inlineStr">
+        <is>
+          <t>funding_cut_pct</t>
+        </is>
+      </c>
+      <c r="B39" s="11" t="inlineStr">
+        <is>
+          <t>Funding reduction</t>
+        </is>
+      </c>
+      <c r="C39" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D39" s="10" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E39" s="10" t="inlineStr">
+        <is>
+          <t>0.0 – 0.6</t>
+        </is>
+      </c>
+      <c r="F39" s="11" t="inlineStr">
+        <is>
+          <t>Scenario lever for a grant reduction or donor hold</t>
+        </is>
+      </c>
+      <c r="G39" s="10" t="inlineStr">
+        <is>
+          <t>Finance &amp; Grants</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="10" t="inlineStr">
+        <is>
+          <t>budget_growth_pct</t>
+        </is>
+      </c>
+      <c r="B40" s="11" t="inlineStr">
+        <is>
+          <t>Budget growth / reallocation</t>
+        </is>
+      </c>
+      <c r="C40" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D40" s="10" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E40" s="10" t="inlineStr">
+        <is>
+          <t>-0.3 – 0.5</t>
+        </is>
+      </c>
+      <c r="F40" s="11" t="inlineStr">
+        <is>
+          <t>Approved additional budget or internal reallocation</t>
+        </is>
+      </c>
+      <c r="G40" s="10" t="inlineStr">
+        <is>
+          <t>Finance &amp; Grants</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="10" t="inlineStr">
+        <is>
+          <t>excess_stock_release_pct</t>
+        </is>
+      </c>
+      <c r="B41" s="11" t="inlineStr">
+        <is>
+          <t>Excess stock used instead of buying</t>
+        </is>
+      </c>
+      <c r="C41" s="12" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="D41" s="10" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E41" s="10" t="inlineStr">
+        <is>
+          <t>0.0 – 1.0</t>
+        </is>
+      </c>
+      <c r="F41" s="11" t="inlineStr">
+        <is>
+          <t>Share of stock held above the target cover that offsets new purchases (redistribution or planned drawdown)</t>
+        </is>
+      </c>
+      <c r="G41" s="10" t="inlineStr">
+        <is>
+          <t>Supply chain</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="10" t="inlineStr">
+        <is>
+          <t>order_cycle_days</t>
+        </is>
+      </c>
+      <c r="B42" s="11" t="inlineStr">
+        <is>
+          <t>Purchase cycle length</t>
+        </is>
+      </c>
+      <c r="C42" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="D42" s="10" t="inlineStr">
+        <is>
+          <t>Days</t>
+        </is>
+      </c>
+      <c r="E42" s="10" t="inlineStr">
+        <is>
+          <t>7 – 120</t>
+        </is>
+      </c>
+      <c r="F42" s="11" t="inlineStr">
+        <is>
+          <t>Days between requisition cycles</t>
+        </is>
+      </c>
+      <c r="G42" s="10" t="inlineStr">
+        <is>
+          <t>Procurement</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Change any of these in config/parameters.json and re-run scripts/refresh_all.py to recalculate every status, commentary line and scenario.</t>
         </is>
       </c>
     </row>
@@ -6663,6 +8212,831 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00F2A65A"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>What-if questions – what changes if a driver moves?</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>These questions are answered by the scenario engine in VPT_WhatIf_Analysis.xlsx. Every lever used is a parameter in config/parameters.json, so a scenario can be added or changed without touching code.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>Q ID</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Analytical question</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>Why it matters (decision it supports)</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>Data required</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>How to answer (logic)</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>Output form</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>Trigger / threshold</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>Cadence</t>
+        </is>
+      </c>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="J4" s="9" t="inlineStr">
+        <is>
+          <t>BRD reference</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="46" customHeight="1">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>WF-01</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>What happens to consumption, purchasing and the funding gap if demand rises 20%?</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>Tests whether the budget and the supply chain can absorb a surge before it happens.</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>Demand growth; run-rate; price and policy parameters</t>
+        </is>
+      </c>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>Run the model with demand_growth_pct = 0.20; compare with the baseline scenario</t>
+        </is>
+      </c>
+      <c r="F5" s="11" t="inlineStr">
+        <is>
+          <t>S1 against S0: consumption, purchase requirement, funding gap</t>
+        </is>
+      </c>
+      <c r="G5" s="10" t="inlineStr">
+        <is>
+          <t>Gap above zero</t>
+        </is>
+      </c>
+      <c r="H5" s="10" t="inlineStr">
+        <is>
+          <t>Quarterly / before peak season</t>
+        </is>
+      </c>
+      <c r="I5" s="10" t="inlineStr">
+        <is>
+          <t>Head of Procurement</t>
+        </is>
+      </c>
+      <c r="J5" s="10" t="inlineStr">
+        <is>
+          <t>§11 page spec</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="46" customHeight="1">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>WF-02</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>Can the budget absorb a 15% price shock on medicines and consumables?</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>Price is the second-largest driver of the gap and is outside VPT's control.</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>Price inflation and shock levers; category weights</t>
+        </is>
+      </c>
+      <c r="E6" s="11" t="inlineStr">
+        <is>
+          <t>Run the model with price_shock_pct = 0.15; read the funding gap and utilisation</t>
+        </is>
+      </c>
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>S2: gap, utilisation, price effect</t>
+        </is>
+      </c>
+      <c r="G6" s="10" t="inlineStr">
+        <is>
+          <t>Utilisation above 100%</t>
+        </is>
+      </c>
+      <c r="H6" s="10" t="inlineStr">
+        <is>
+          <t>Quarterly</t>
+        </is>
+      </c>
+      <c r="I6" s="10" t="inlineStr">
+        <is>
+          <t>Finance &amp; Grants</t>
+        </is>
+      </c>
+      <c r="J6" s="10" t="inlineStr">
+        <is>
+          <t>§11 page spec</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="46" customHeight="1">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>WF-03</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>How many items would run out if lead times rose 60% and reliability fell to 70%?</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>Supply disruption is the fastest route from a good plan to a clinical stock-out.</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>Lead-time multiplier; supplier reliability; per-item cover</t>
+        </is>
+      </c>
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>Run the model with the disruption levers; count items whose projected cover is below lead time plus safety stock</t>
+        </is>
+      </c>
+      <c r="F7" s="11" t="inlineStr">
+        <is>
+          <t>S3: stock-out item count and list</t>
+        </is>
+      </c>
+      <c r="G7" s="10" t="inlineStr">
+        <is>
+          <t>Any critical item</t>
+        </is>
+      </c>
+      <c r="H7" s="10" t="inlineStr">
+        <is>
+          <t>Quarterly / when a supplier is at risk</t>
+        </is>
+      </c>
+      <c r="I7" s="10" t="inlineStr">
+        <is>
+          <t>Procurement</t>
+        </is>
+      </c>
+      <c r="J7" s="10" t="inlineStr">
+        <is>
+          <t>§11 page spec</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="46" customHeight="1">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>WF-04</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>What is the exposure if a grant instalment is cut by 20%?</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>Funding shocks are decided elsewhere but must be planned for here.</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>Funding cut lever; consumption and budget</t>
+        </is>
+      </c>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>Run the model with funding_cut_pct = 0.20; read the gap and the utilisation</t>
+        </is>
+      </c>
+      <c r="F8" s="11" t="inlineStr">
+        <is>
+          <t>S4: funding gap, months of cover the budget buys</t>
+        </is>
+      </c>
+      <c r="G8" s="10" t="inlineStr">
+        <is>
+          <t>Gap above materiality</t>
+        </is>
+      </c>
+      <c r="H8" s="10" t="inlineStr">
+        <is>
+          <t>On any donor signal</t>
+        </is>
+      </c>
+      <c r="I8" s="10" t="inlineStr">
+        <is>
+          <t>Finance &amp; Grants</t>
+        </is>
+      </c>
+      <c r="J8" s="10" t="inlineStr">
+        <is>
+          <t>§11 page spec</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="46" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>WF-05</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>How much cash is released if we move from 90 to 60 days of cover?</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>Cover policy is the most direct lever management controls.</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>Target cover; safety stock; excess stock release</t>
+        </is>
+      </c>
+      <c r="E9" s="11" t="inlineStr">
+        <is>
+          <t>Run the model at several cover levels; read working capital and purchase requirement</t>
+        </is>
+      </c>
+      <c r="F9" s="11" t="inlineStr">
+        <is>
+          <t>S5 and the cover trade-off curve</t>
+        </is>
+      </c>
+      <c r="G9" s="10" t="inlineStr">
+        <is>
+          <t>Capital release above PKR 5m</t>
+        </is>
+      </c>
+      <c r="H9" s="10" t="inlineStr">
+        <is>
+          <t>Twice yearly</t>
+        </is>
+      </c>
+      <c r="I9" s="10" t="inlineStr">
+        <is>
+          <t>Head of Procurement</t>
+        </is>
+      </c>
+      <c r="J9" s="10" t="inlineStr">
+        <is>
+          <t>§11 page spec</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="46" customHeight="1">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>WF-06</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>What is the effect of a framework contract at 8% below current prices?</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>Tests whether commercial action alone can close the gap.</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>Bulk discount; lead time; supplier reliability</t>
+        </is>
+      </c>
+      <c r="E10" s="11" t="inlineStr">
+        <is>
+          <t>Run the model with bulk_discount_pct = 0.08 and improved supply assumptions</t>
+        </is>
+      </c>
+      <c r="F10" s="11" t="inlineStr">
+        <is>
+          <t>S6: purchase value, ratio, gap</t>
+        </is>
+      </c>
+      <c r="G10" s="10" t="inlineStr">
+        <is>
+          <t>Gap reduction</t>
+        </is>
+      </c>
+      <c r="H10" s="10" t="inlineStr">
+        <is>
+          <t>Before the contract cycle</t>
+        </is>
+      </c>
+      <c r="I10" s="10" t="inlineStr">
+        <is>
+          <t>Procurement</t>
+        </is>
+      </c>
+      <c r="J10" s="10" t="inlineStr">
+        <is>
+          <t>§11 page spec</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="46" customHeight="1">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>WF-07</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>What is the combined downside if everything moves against us at once?</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>Single shocks are survivable; correlated shocks are not.</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>Demand, price, lead time, reliability and funding levers together</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="inlineStr">
+        <is>
+          <t>Run the combined-lever scenario; compare with S0 and with the single-shock cases</t>
+        </is>
+      </c>
+      <c r="F11" s="11" t="inlineStr">
+        <is>
+          <t>S7: gap, purchase, stock-outs, expiry</t>
+        </is>
+      </c>
+      <c r="G11" s="10" t="inlineStr">
+        <is>
+          <t>Any projection beyond tolerance</t>
+        </is>
+      </c>
+      <c r="H11" s="10" t="inlineStr">
+        <is>
+          <t>Quarterly</t>
+        </is>
+      </c>
+      <c r="I11" s="10" t="inlineStr">
+        <is>
+          <t>Business owner</t>
+        </is>
+      </c>
+      <c r="J11" s="10" t="inlineStr">
+        <is>
+          <t>§11 page spec</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="46" customHeight="1">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>WF-08</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>How much of that downside can we absorb with the levers we control?</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>Separates the unavoidable part of a shock from the part management can manage.</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>Policy and commercial levers applied on top of the downside</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="inlineStr">
+        <is>
+          <t>Run the optimised-response scenario; take the difference against the downside</t>
+        </is>
+      </c>
+      <c r="F12" s="11" t="inlineStr">
+        <is>
+          <t>S8 vs S7: gap, purchase and stock-out reduction</t>
+        </is>
+      </c>
+      <c r="G12" s="10" t="inlineStr">
+        <is>
+          <t>Residual gap remains</t>
+        </is>
+      </c>
+      <c r="H12" s="10" t="inlineStr">
+        <is>
+          <t>Quarterly</t>
+        </is>
+      </c>
+      <c r="I12" s="10" t="inlineStr">
+        <is>
+          <t>Business owner</t>
+        </is>
+      </c>
+      <c r="J12" s="10" t="inlineStr">
+        <is>
+          <t>§11 page spec</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="46" customHeight="1">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>WF-09</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>Which parameter should we watch most closely?</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>Monitoring effort should follow the size of the effect, not the ease of measurement.</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>Sensitivity ranges and all model outputs</t>
+        </is>
+      </c>
+      <c r="E13" s="11" t="inlineStr">
+        <is>
+          <t>Move each lever between its low and high value and rank by swing (tornado)</t>
+        </is>
+      </c>
+      <c r="F13" s="11" t="inlineStr">
+        <is>
+          <t>06_Sensitivity ranking</t>
+        </is>
+      </c>
+      <c r="G13" s="10" t="inlineStr">
+        <is>
+          <t>Swing above 10% of the output</t>
+        </is>
+      </c>
+      <c r="H13" s="10" t="inlineStr">
+        <is>
+          <t>Quarterly</t>
+        </is>
+      </c>
+      <c r="I13" s="10" t="inlineStr">
+        <is>
+          <t>Business analyst</t>
+        </is>
+      </c>
+      <c r="J13" s="10" t="inlineStr">
+        <is>
+          <t>§11 page spec</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="46" customHeight="1">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>WF-10</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>How far can price or demand move before the budget breaks?</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>Converts the budget position into a tolerance the business can watch.</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>Break-even solve on price inflation and demand growth</t>
+        </is>
+      </c>
+      <c r="E14" s="11" t="inlineStr">
+        <is>
+          <t>Solve for the lever value at which the funding gap becomes zero</t>
+        </is>
+      </c>
+      <c r="F14" s="11" t="inlineStr">
+        <is>
+          <t>07_BreakEven</t>
+        </is>
+      </c>
+      <c r="G14" s="10" t="inlineStr">
+        <is>
+          <t>Break-even inside the plausible range</t>
+        </is>
+      </c>
+      <c r="H14" s="10" t="inlineStr">
+        <is>
+          <t>Quarterly</t>
+        </is>
+      </c>
+      <c r="I14" s="10" t="inlineStr">
+        <is>
+          <t>Finance &amp; Grants</t>
+        </is>
+      </c>
+      <c r="J14" s="10" t="inlineStr">
+        <is>
+          <t>§11 page spec</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="46" customHeight="1">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>WF-11</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>What is the right stock-cover policy?</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>Cover is a trade-off between working capital, purchase cost and stock-out risk.</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>Cover trade-off curve (30–210 days)</t>
+        </is>
+      </c>
+      <c r="E15" s="11" t="inlineStr">
+        <is>
+          <t>Read purchase requirement, expiry risk and working capital across the cover range; choose at the knee of the curve</t>
+        </is>
+      </c>
+      <c r="F15" s="11" t="inlineStr">
+        <is>
+          <t>07_BreakEven trade-off curve</t>
+        </is>
+      </c>
+      <c r="G15" s="10" t="inlineStr">
+        <is>
+          <t>Expiry or stock-out above tolerance</t>
+        </is>
+      </c>
+      <c r="H15" s="10" t="inlineStr">
+        <is>
+          <t>Twice yearly</t>
+        </is>
+      </c>
+      <c r="I15" s="10" t="inlineStr">
+        <is>
+          <t>Head of Procurement</t>
+        </is>
+      </c>
+      <c r="J15" s="10" t="inlineStr">
+        <is>
+          <t>§11 page spec</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="46" customHeight="1">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>WF-12</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>Which combination of demand growth and inflation puts us over budget?</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>Gives a map rather than a single point, so unplanned combinations are visible.</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>Two-way table over demand and price</t>
+        </is>
+      </c>
+      <c r="E16" s="11" t="inlineStr">
+        <is>
+          <t>Read the grid for funding gap and utilisation; locate the current position</t>
+        </is>
+      </c>
+      <c r="F16" s="11" t="inlineStr">
+        <is>
+          <t>08_TwoWay</t>
+        </is>
+      </c>
+      <c r="G16" s="10" t="inlineStr">
+        <is>
+          <t>Any red cell in the plausible range</t>
+        </is>
+      </c>
+      <c r="H16" s="10" t="inlineStr">
+        <is>
+          <t>Quarterly</t>
+        </is>
+      </c>
+      <c r="I16" s="10" t="inlineStr">
+        <is>
+          <t>Finance &amp; Grants</t>
+        </is>
+      </c>
+      <c r="J16" s="10" t="inlineStr">
+        <is>
+          <t>§11 page spec</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="46" customHeight="1">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>WF-13</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>What if a project ends earlier than planned, or a new project starts mid-year?</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>Portfolio changes move every projection; they are not gradual.</t>
+        </is>
+      </c>
+      <c r="D17" s="11" t="inlineStr">
+        <is>
+          <t>Activity factor; project start and end dates</t>
+        </is>
+      </c>
+      <c r="E17" s="11" t="inlineStr">
+        <is>
+          <t>Adjust activity_factor for the share of the year the portfolio is active; rerun</t>
+        </is>
+      </c>
+      <c r="F17" s="11" t="inlineStr">
+        <is>
+          <t>Scenario variant of S0</t>
+        </is>
+      </c>
+      <c r="G17" s="10" t="inlineStr">
+        <is>
+          <t>Activity factor change above 10%</t>
+        </is>
+      </c>
+      <c r="H17" s="10" t="inlineStr">
+        <is>
+          <t>On any portfolio change</t>
+        </is>
+      </c>
+      <c r="I17" s="10" t="inlineStr">
+        <is>
+          <t>Programme</t>
+        </is>
+      </c>
+      <c r="J17" s="10" t="inlineStr">
+        <is>
+          <t>§11 page spec</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="46" customHeight="1">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>WF-14</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>What should we change now so that the downside scenario does not become the baseline?</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>The purpose of all of the above: a decision, not a projection.</t>
+        </is>
+      </c>
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>All levers, compared across scenarios</t>
+        </is>
+      </c>
+      <c r="E18" s="11" t="inlineStr">
+        <is>
+          <t>Identify the levers with the largest gap reduction at acceptable cost and risk; convert into actions with owners</t>
+        </is>
+      </c>
+      <c r="F18" s="11" t="inlineStr">
+        <is>
+          <t>Action plan from S8 vs S7</t>
+        </is>
+      </c>
+      <c r="G18" s="10" t="inlineStr">
+        <is>
+          <t>Residual gap above materiality</t>
+        </is>
+      </c>
+      <c r="H18" s="10" t="inlineStr">
+        <is>
+          <t>Quarterly</t>
+        </is>
+      </c>
+      <c r="I18" s="10" t="inlineStr">
+        <is>
+          <t>Business owner</t>
+        </is>
+      </c>
+      <c r="J18" s="10" t="inlineStr">
+        <is>
+          <t>§11 page spec</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:J18"/>
+  <mergeCells count="1">
+    <mergeCell ref="A2:J2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="0072B7B2"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -6758,7 +9132,7 @@
           <t>Total consumption value in the period</t>
         </is>
       </c>
-      <c r="D5" s="13" t="n">
+      <c r="D5" s="14" t="n">
         <v>261575946.1</v>
       </c>
       <c r="E5" s="10" t="inlineStr">
@@ -6771,7 +9145,7 @@
           <t>Report</t>
         </is>
       </c>
-      <c r="G5" s="14" t="inlineStr">
+      <c r="G5" s="15" t="inlineStr">
         <is>
           <t>Info</t>
         </is>
@@ -6803,7 +9177,7 @@
           <t>Procurement investment (excl. cancelled)</t>
         </is>
       </c>
-      <c r="D6" s="13" t="n">
+      <c r="D6" s="14" t="n">
         <v>300845059.6</v>
       </c>
       <c r="E6" s="10" t="inlineStr">
@@ -6816,7 +9190,7 @@
           <t>Report</t>
         </is>
       </c>
-      <c r="G6" s="14" t="inlineStr">
+      <c r="G6" s="15" t="inlineStr">
         <is>
           <t>Info</t>
         </is>
@@ -6848,7 +9222,7 @@
           <t>Open commitment (ordered, not received)</t>
         </is>
       </c>
-      <c r="D7" s="13" t="n">
+      <c r="D7" s="14" t="n">
         <v>4467950.63</v>
       </c>
       <c r="E7" s="10" t="inlineStr">
@@ -6861,7 +9235,7 @@
           <t>Trend down</t>
         </is>
       </c>
-      <c r="G7" s="15" t="inlineStr">
+      <c r="G7" s="16" t="inlineStr">
         <is>
           <t>Green</t>
         </is>
@@ -6893,7 +9267,7 @@
           <t>Consumption-to-investment ratio (period)</t>
         </is>
       </c>
-      <c r="D8" s="16" t="n">
+      <c r="D8" s="13" t="n">
         <v>0.869</v>
       </c>
       <c r="E8" s="10" t="inlineStr">
@@ -6906,7 +9280,7 @@
           <t>0.80 – 1.05</t>
         </is>
       </c>
-      <c r="G8" s="15" t="inlineStr">
+      <c r="G8" s="16" t="inlineStr">
         <is>
           <t>Green</t>
         </is>
@@ -6938,7 +9312,7 @@
           <t>Largest consuming project – share of total (Maternal &amp; Child Health Prog)</t>
         </is>
       </c>
-      <c r="D9" s="17" t="n">
+      <c r="D9" s="12" t="n">
         <v>0.232</v>
       </c>
       <c r="E9" s="10" t="inlineStr">
@@ -6951,7 +9325,7 @@
           <t>Concentration monitor</t>
         </is>
       </c>
-      <c r="G9" s="14" t="inlineStr">
+      <c r="G9" s="15" t="inlineStr">
         <is>
           <t>Info</t>
         </is>
@@ -6983,7 +9357,7 @@
           <t>Share of consumption value held by the top 10 items</t>
         </is>
       </c>
-      <c r="D10" s="17" t="n">
+      <c r="D10" s="12" t="n">
         <v>0.457</v>
       </c>
       <c r="E10" s="10" t="inlineStr">
@@ -6996,7 +9370,7 @@
           <t>Monitor</t>
         </is>
       </c>
-      <c r="G10" s="14" t="inlineStr">
+      <c r="G10" s="15" t="inlineStr">
         <is>
           <t>Info</t>
         </is>
@@ -7028,7 +9402,7 @@
           <t>Items required to reach 80% of consumption value (of 83)</t>
         </is>
       </c>
-      <c r="D11" s="13" t="n">
+      <c r="D11" s="14" t="n">
         <v>32</v>
       </c>
       <c r="E11" s="10" t="inlineStr">
@@ -7041,7 +9415,7 @@
           <t>Pareto</t>
         </is>
       </c>
-      <c r="G11" s="14" t="inlineStr">
+      <c r="G11" s="15" t="inlineStr">
         <is>
           <t>Info</t>
         </is>
@@ -7088,7 +9462,7 @@
           <t>vs avg +52%</t>
         </is>
       </c>
-      <c r="G12" s="14" t="inlineStr">
+      <c r="G12" s="15" t="inlineStr">
         <is>
           <t>Info</t>
         </is>
@@ -7120,7 +9494,7 @@
           <t>Year-on-year consumption growth (FY2025-26 vs FY2024-25)</t>
         </is>
       </c>
-      <c r="D13" s="17" t="n">
+      <c r="D13" s="12" t="n">
         <v>0.215</v>
       </c>
       <c r="E13" s="10" t="inlineStr">
@@ -7133,7 +9507,7 @@
           <t>±10%</t>
         </is>
       </c>
-      <c r="G13" s="15" t="inlineStr">
+      <c r="G13" s="16" t="inlineStr">
         <is>
           <t>Green</t>
         </is>
@@ -7165,7 +9539,7 @@
           <t>Stock on hand value at report date</t>
         </is>
       </c>
-      <c r="D14" s="13" t="n">
+      <c r="D14" s="14" t="n">
         <v>41090443.94</v>
       </c>
       <c r="E14" s="10" t="inlineStr">
@@ -7178,7 +9552,7 @@
           <t>Report</t>
         </is>
       </c>
-      <c r="G14" s="14" t="inlineStr">
+      <c r="G14" s="15" t="inlineStr">
         <is>
           <t>Info</t>
         </is>
@@ -7210,7 +9584,7 @@
           <t>Items with less than 60 days of cover</t>
         </is>
       </c>
-      <c r="D15" s="13" t="n">
+      <c r="D15" s="14" t="n">
         <v>3</v>
       </c>
       <c r="E15" s="10" t="inlineStr">
@@ -7223,7 +9597,7 @@
           <t>0 critical</t>
         </is>
       </c>
-      <c r="G15" s="15" t="inlineStr">
+      <c r="G15" s="16" t="inlineStr">
         <is>
           <t>Green</t>
         </is>
@@ -7270,7 +9644,7 @@
           <t>32 days</t>
         </is>
       </c>
-      <c r="G16" s="18" t="inlineStr">
+      <c r="G16" s="17" t="inlineStr">
         <is>
           <t>Red</t>
         </is>
@@ -7302,7 +9676,7 @@
           <t>Stock value with more than 180 days of cover</t>
         </is>
       </c>
-      <c r="D17" s="13" t="n">
+      <c r="D17" s="14" t="n">
         <v>3446230</v>
       </c>
       <c r="E17" s="10" t="inlineStr">
@@ -7315,7 +9689,7 @@
           <t>Freeze re-order</t>
         </is>
       </c>
-      <c r="G17" s="18" t="inlineStr">
+      <c r="G17" s="17" t="inlineStr">
         <is>
           <t>Red</t>
         </is>
@@ -7347,7 +9721,7 @@
           <t>Expired stock held (value)</t>
         </is>
       </c>
-      <c r="D18" s="13" t="n">
+      <c r="D18" s="14" t="n">
         <v>783764.1800000001</v>
       </c>
       <c r="E18" s="10" t="inlineStr">
@@ -7360,7 +9734,7 @@
           <t>Zero</t>
         </is>
       </c>
-      <c r="G18" s="18" t="inlineStr">
+      <c r="G18" s="17" t="inlineStr">
         <is>
           <t>Red</t>
         </is>
@@ -7392,7 +9766,7 @@
           <t>Stock expiring within 60 days (value)</t>
         </is>
       </c>
-      <c r="D19" s="13" t="n">
+      <c r="D19" s="14" t="n">
         <v>950939.91</v>
       </c>
       <c r="E19" s="10" t="inlineStr">
@@ -7405,7 +9779,7 @@
           <t>Minimise</t>
         </is>
       </c>
-      <c r="G19" s="18" t="inlineStr">
+      <c r="G19" s="17" t="inlineStr">
         <is>
           <t>Red</t>
         </is>
@@ -7437,7 +9811,7 @@
           <t>Slow / non-moving items (count)</t>
         </is>
       </c>
-      <c r="D20" s="13" t="n">
+      <c r="D20" s="14" t="n">
         <v>5</v>
       </c>
       <c r="E20" s="10" t="inlineStr">
@@ -7450,7 +9824,7 @@
           <t>Minimise</t>
         </is>
       </c>
-      <c r="G20" s="18" t="inlineStr">
+      <c r="G20" s="17" t="inlineStr">
         <is>
           <t>Red</t>
         </is>
@@ -7482,7 +9856,7 @@
           <t>Slow / non-moving stock value</t>
         </is>
       </c>
-      <c r="D21" s="13" t="n">
+      <c r="D21" s="14" t="n">
         <v>168300</v>
       </c>
       <c r="E21" s="10" t="inlineStr">
@@ -7495,7 +9869,7 @@
           <t>Minimise</t>
         </is>
       </c>
-      <c r="G21" s="15" t="inlineStr">
+      <c r="G21" s="16" t="inlineStr">
         <is>
           <t>Green</t>
         </is>
@@ -7527,7 +9901,7 @@
           <t>Number of PO lines with an open balance</t>
         </is>
       </c>
-      <c r="D22" s="13" t="n">
+      <c r="D22" s="14" t="n">
         <v>320</v>
       </c>
       <c r="E22" s="10" t="inlineStr">
@@ -7540,7 +9914,7 @@
           <t>Trend down</t>
         </is>
       </c>
-      <c r="G22" s="14" t="inlineStr">
+      <c r="G22" s="15" t="inlineStr">
         <is>
           <t>Info</t>
         </is>
@@ -7572,7 +9946,7 @@
           <t>Cancelled purchase order lines</t>
         </is>
       </c>
-      <c r="D23" s="13" t="n">
+      <c r="D23" s="14" t="n">
         <v>847</v>
       </c>
       <c r="E23" s="10" t="inlineStr">
@@ -7585,7 +9959,7 @@
           <t>&lt; 2% of lines</t>
         </is>
       </c>
-      <c r="G23" s="18" t="inlineStr">
+      <c r="G23" s="17" t="inlineStr">
         <is>
           <t>Red</t>
         </is>
@@ -7617,7 +9991,7 @@
           <t>Average unit price movement, first vs latest purchase</t>
         </is>
       </c>
-      <c r="D24" s="17" t="n">
+      <c r="D24" s="12" t="n">
         <v>0.162</v>
       </c>
       <c r="E24" s="10" t="inlineStr">
@@ -7630,7 +10004,7 @@
           <t>&lt; 10%</t>
         </is>
       </c>
-      <c r="G24" s="18" t="inlineStr">
+      <c r="G24" s="17" t="inlineStr">
         <is>
           <t>Red</t>
         </is>
@@ -7662,7 +10036,7 @@
           <t>Cost per beneficiary for the period</t>
         </is>
       </c>
-      <c r="D25" s="13" t="n">
+      <c r="D25" s="14" t="n">
         <v>384.81</v>
       </c>
       <c r="E25" s="10" t="inlineStr">
@@ -7675,7 +10049,7 @@
           <t>Peer band</t>
         </is>
       </c>
-      <c r="G25" s="14" t="inlineStr">
+      <c r="G25" s="15" t="inlineStr">
         <is>
           <t>Info</t>
         </is>
@@ -7707,7 +10081,7 @@
           <t>Spread between the highest and lowest project cost per beneficiary</t>
         </is>
       </c>
-      <c r="D26" s="17" t="n">
+      <c r="D26" s="12" t="n">
         <v>1.208</v>
       </c>
       <c r="E26" s="10" t="inlineStr">
@@ -7720,7 +10094,7 @@
           <t>&lt; 30%</t>
         </is>
       </c>
-      <c r="G26" s="18" t="inlineStr">
+      <c r="G26" s="17" t="inlineStr">
         <is>
           <t>Red</t>
         </is>
@@ -7752,7 +10126,7 @@
           <t>Product budget utilisation for the period</t>
         </is>
       </c>
-      <c r="D27" s="17" t="n">
+      <c r="D27" s="12" t="n">
         <v>0.764</v>
       </c>
       <c r="E27" s="10" t="inlineStr">
@@ -7765,7 +10139,7 @@
           <t>In line with elapsed time</t>
         </is>
       </c>
-      <c r="G27" s="15" t="inlineStr">
+      <c r="G27" s="16" t="inlineStr">
         <is>
           <t>Green</t>
         </is>
@@ -7797,7 +10171,7 @@
           <t>Unattributed consumption as a share of value</t>
         </is>
       </c>
-      <c r="D28" s="17" t="n">
+      <c r="D28" s="12" t="n">
         <v>0.024</v>
       </c>
       <c r="E28" s="10" t="inlineStr">
@@ -7810,7 +10184,7 @@
           <t>≤ 1.0%</t>
         </is>
       </c>
-      <c r="G28" s="18" t="inlineStr">
+      <c r="G28" s="17" t="inlineStr">
         <is>
           <t>Red</t>
         </is>
@@ -7842,7 +10216,7 @@
           <t>Projects ending within 120 days with unspent budget</t>
         </is>
       </c>
-      <c r="D29" s="13" t="n">
+      <c r="D29" s="14" t="n">
         <v>6</v>
       </c>
       <c r="E29" s="10" t="inlineStr">
@@ -7855,7 +10229,7 @@
           <t>0 unmanaged</t>
         </is>
       </c>
-      <c r="G29" s="18" t="inlineStr">
+      <c r="G29" s="17" t="inlineStr">
         <is>
           <t>Red</t>
         </is>
@@ -7887,7 +10261,7 @@
           <t>Latest month (Sep-2026) vs preceding 3-month average</t>
         </is>
       </c>
-      <c r="D30" s="17" t="n">
+      <c r="D30" s="12" t="n">
         <v>0.045</v>
       </c>
       <c r="E30" s="10" t="inlineStr">
@@ -7900,7 +10274,7 @@
           <t>±15%</t>
         </is>
       </c>
-      <c r="G30" s="15" t="inlineStr">
+      <c r="G30" s="16" t="inlineStr">
         <is>
           <t>Green</t>
         </is>
@@ -7932,7 +10306,7 @@
           <t>Expense categories over budget</t>
         </is>
       </c>
-      <c r="D31" s="13" t="n">
+      <c r="D31" s="14" t="n">
         <v>3</v>
       </c>
       <c r="E31" s="10" t="inlineStr">
@@ -7945,7 +10319,7 @@
           <t>0</t>
         </is>
       </c>
-      <c r="G31" s="18" t="inlineStr">
+      <c r="G31" s="17" t="inlineStr">
         <is>
           <t>Red</t>
         </is>
@@ -7992,7 +10366,7 @@
           <t>≤ 100%</t>
         </is>
       </c>
-      <c r="G32" s="18" t="inlineStr">
+      <c r="G32" s="17" t="inlineStr">
         <is>
           <t>Red</t>
         </is>
@@ -8039,7 +10413,7 @@
           <t>≤ 1%</t>
         </is>
       </c>
-      <c r="G33" s="18" t="inlineStr">
+      <c r="G33" s="17" t="inlineStr">
         <is>
           <t>Red</t>
         </is>
@@ -8071,7 +10445,7 @@
           <t>Items with price increase above 10%</t>
         </is>
       </c>
-      <c r="D34" s="13" t="n">
+      <c r="D34" s="14" t="n">
         <v>5</v>
       </c>
       <c r="E34" s="10" t="inlineStr">
@@ -8084,7 +10458,7 @@
           <t>0</t>
         </is>
       </c>
-      <c r="G34" s="18" t="inlineStr">
+      <c r="G34" s="17" t="inlineStr">
         <is>
           <t>Red</t>
         </is>
@@ -8116,7 +10490,7 @@
           <t>Duplicate receipt candidates</t>
         </is>
       </c>
-      <c r="D35" s="13" t="n">
+      <c r="D35" s="14" t="n">
         <v>8</v>
       </c>
       <c r="E35" s="10" t="inlineStr">
@@ -8129,7 +10503,7 @@
           <t>0</t>
         </is>
       </c>
-      <c r="G35" s="18" t="inlineStr">
+      <c r="G35" s="17" t="inlineStr">
         <is>
           <t>Red</t>
         </is>
@@ -8176,7 +10550,7 @@
           <t>Within 2σ</t>
         </is>
       </c>
-      <c r="G36" s="14" t="inlineStr">
+      <c r="G36" s="15" t="inlineStr">
         <is>
           <t>Info</t>
         </is>
@@ -8208,7 +10582,7 @@
           <t>Projected consumption – next 3 months (run rate)</t>
         </is>
       </c>
-      <c r="D37" s="13" t="n">
+      <c r="D37" s="14" t="n">
         <v>33768376.88</v>
       </c>
       <c r="E37" s="10" t="inlineStr">
@@ -8221,7 +10595,7 @@
           <t>Within budget trajectory</t>
         </is>
       </c>
-      <c r="G37" s="14" t="inlineStr">
+      <c r="G37" s="15" t="inlineStr">
         <is>
           <t>Info</t>
         </is>
@@ -8253,8 +10627,8 @@
           <t>Projected consumption – full FY2026-27 (straight line)</t>
         </is>
       </c>
-      <c r="D38" s="13" t="n">
-        <v>135073507.52</v>
+      <c r="D38" s="14" t="n">
+        <v>67536753.76000001</v>
       </c>
       <c r="E38" s="10" t="inlineStr">
         <is>
@@ -8266,7 +10640,7 @@
           <t>Budget 67,078,000</t>
         </is>
       </c>
-      <c r="G38" s="18" t="inlineStr">
+      <c r="G38" s="17" t="inlineStr">
         <is>
           <t>Red</t>
         </is>
@@ -8298,7 +10672,7 @@
           <t>Items likely to breach 30 days cover before next delivery</t>
         </is>
       </c>
-      <c r="D39" s="13" t="n">
+      <c r="D39" s="14" t="n">
         <v>0</v>
       </c>
       <c r="E39" s="10" t="inlineStr">
@@ -8311,7 +10685,7 @@
           <t>0</t>
         </is>
       </c>
-      <c r="G39" s="15" t="inlineStr">
+      <c r="G39" s="16" t="inlineStr">
         <is>
           <t>Green</t>
         </is>
@@ -8343,7 +10717,7 @@
           <t>Value expected to expire within 60 days at current consumption</t>
         </is>
       </c>
-      <c r="D40" s="13" t="n">
+      <c r="D40" s="14" t="n">
         <v>950939.91</v>
       </c>
       <c r="E40" s="10" t="inlineStr">
@@ -8356,7 +10730,7 @@
           <t>Minimise</t>
         </is>
       </c>
-      <c r="G40" s="18" t="inlineStr">
+      <c r="G40" s="17" t="inlineStr">
         <is>
           <t>Red</t>
         </is>
@@ -8388,7 +10762,7 @@
           <t>Unspent budget exposure in projects ending within 120 days</t>
         </is>
       </c>
-      <c r="D41" s="13" t="n">
+      <c r="D41" s="14" t="n">
         <v>136478186.83</v>
       </c>
       <c r="E41" s="10" t="inlineStr">
@@ -8401,7 +10775,7 @@
           <t>Minimise</t>
         </is>
       </c>
-      <c r="G41" s="18" t="inlineStr">
+      <c r="G41" s="17" t="inlineStr">
         <is>
           <t>Red</t>
         </is>
@@ -8433,7 +10807,7 @@
           <t>Number of projects projected to exceed budget</t>
         </is>
       </c>
-      <c r="D42" s="13" t="n">
+      <c r="D42" s="14" t="n">
         <v>0</v>
       </c>
       <c r="E42" s="10" t="inlineStr">
@@ -8446,7 +10820,7 @@
           <t>0</t>
         </is>
       </c>
-      <c r="G42" s="15" t="inlineStr">
+      <c r="G42" s="16" t="inlineStr">
         <is>
           <t>Green</t>
         </is>
@@ -8478,8 +10852,8 @@
           <t>Additional budget needed to hold service levels to year end</t>
         </is>
       </c>
-      <c r="D43" s="13" t="n">
-        <v>67995507.52</v>
+      <c r="D43" s="14" t="n">
+        <v>458753.76</v>
       </c>
       <c r="E43" s="10" t="inlineStr">
         <is>
@@ -8491,7 +10865,7 @@
           <t>0</t>
         </is>
       </c>
-      <c r="G43" s="18" t="inlineStr">
+      <c r="G43" s="17" t="inlineStr">
         <is>
           <t>Red</t>
         </is>
@@ -8523,7 +10897,7 @@
           <t>Redistribution opportunities (surplus cover matched to deficit)</t>
         </is>
       </c>
-      <c r="D44" s="13" t="n">
+      <c r="D44" s="14" t="n">
         <v>10</v>
       </c>
       <c r="E44" s="10" t="inlineStr">
@@ -8536,7 +10910,7 @@
           <t>Maximise</t>
         </is>
       </c>
-      <c r="G44" s="14" t="inlineStr">
+      <c r="G44" s="15" t="inlineStr">
         <is>
           <t>Info</t>
         </is>
@@ -8568,7 +10942,7 @@
           <t>Items in the current requirement proposal</t>
         </is>
       </c>
-      <c r="D45" s="13" t="n">
+      <c r="D45" s="14" t="n">
         <v>10</v>
       </c>
       <c r="E45" s="10" t="inlineStr">
@@ -8581,7 +10955,7 @@
           <t>Reviewed monthly</t>
         </is>
       </c>
-      <c r="G45" s="14" t="inlineStr">
+      <c r="G45" s="15" t="inlineStr">
         <is>
           <t>Info</t>
         </is>
@@ -8613,7 +10987,7 @@
           <t>Critical items requiring immediate action</t>
         </is>
       </c>
-      <c r="D46" s="13" t="n">
+      <c r="D46" s="14" t="n">
         <v>0</v>
       </c>
       <c r="E46" s="10" t="inlineStr">
@@ -8626,7 +11000,7 @@
           <t>0</t>
         </is>
       </c>
-      <c r="G46" s="15" t="inlineStr">
+      <c r="G46" s="16" t="inlineStr">
         <is>
           <t>Green</t>
         </is>
@@ -8658,7 +11032,7 @@
           <t>Master-data corrections outstanding</t>
         </is>
       </c>
-      <c r="D47" s="13" t="n">
+      <c r="D47" s="14" t="n">
         <v>3</v>
       </c>
       <c r="E47" s="10" t="inlineStr">
@@ -8671,7 +11045,7 @@
           <t>0</t>
         </is>
       </c>
-      <c r="G47" s="18" t="inlineStr">
+      <c r="G47" s="17" t="inlineStr">
         <is>
           <t>Red</t>
         </is>
@@ -8718,7 +11092,7 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="G48" s="15" t="inlineStr">
+      <c r="G48" s="16" t="inlineStr">
         <is>
           <t>Green</t>
         </is>
@@ -8750,7 +11124,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00F2A65A"/>
@@ -9209,836 +11583,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="00E45756"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:J20"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="58" customWidth="1" min="6" max="6"/>
-    <col width="46" customWidth="1" min="7" max="7"/>
-    <col width="52" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Live data commentary – what happened, why, so what, now what, when, who</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Generated from the data as at 2026-09-30. Each line is produced only because the metric breached its threshold in 01_Parameters; on refresh, lines move between Red, Amber and Green automatically.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="32" customHeight="1">
-      <c r="A4" s="9" t="inlineStr">
-        <is>
-          <t>Ref</t>
-        </is>
-      </c>
-      <c r="B4" s="9" t="inlineStr">
-        <is>
-          <t>Metric</t>
-        </is>
-      </c>
-      <c r="C4" s="9" t="inlineStr">
-        <is>
-          <t>Current value</t>
-        </is>
-      </c>
-      <c r="D4" s="9" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="E4" s="9" t="inlineStr">
-        <is>
-          <t>What happened (data)</t>
-        </is>
-      </c>
-      <c r="F4" s="9" t="inlineStr">
-        <is>
-          <t>Why it happened – causes to test</t>
-        </is>
-      </c>
-      <c r="G4" s="9" t="inlineStr">
-        <is>
-          <t>So what (impact)</t>
-        </is>
-      </c>
-      <c r="H4" s="9" t="inlineStr">
-        <is>
-          <t>What to do (action)</t>
-        </is>
-      </c>
-      <c r="I4" s="9" t="inlineStr">
-        <is>
-          <t>When to act</t>
-        </is>
-      </c>
-      <c r="J4" s="9" t="inlineStr">
-        <is>
-          <t>Owner / escalate</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="132" customHeight="1">
-      <c r="A5" s="10" t="inlineStr">
-        <is>
-          <t>CM-01</t>
-        </is>
-      </c>
-      <c r="B5" s="11" t="inlineStr">
-        <is>
-          <t>Consumption-to-investment ratio</t>
-        </is>
-      </c>
-      <c r="C5" s="11" t="inlineStr">
-        <is>
-          <t>0.87</t>
-        </is>
-      </c>
-      <c r="D5" s="19" t="inlineStr">
-        <is>
-          <t>Green</t>
-        </is>
-      </c>
-      <c r="E5" s="11" t="inlineStr">
-        <is>
-          <t>Consumption of PKR 261,575,946 against investment of PKR 300,845,060 gives a ratio of 0.87 for the period.</t>
-        </is>
-      </c>
-      <c r="F5" s="11" t="inlineStr">
-        <is>
-          <t>Ranked causes to test: (1) ordering ahead of need due to pack sizes or bulk discounts; (2) project start-up stock build; (3) slow issuing at service points; (4) drawdown of opening stock with no new purchase; (5) delayed receipts moving investment into a later period.</t>
-        </is>
-      </c>
-      <c r="G5" s="11" t="inlineStr">
-        <is>
-          <t>Value purchased but not yet used is cash tied up in store and at risk of expiry; a ratio far above 1.05 means consumption is being funded from stock and a stock-out will follow.</t>
-        </is>
-      </c>
-      <c r="H5" s="11" t="inlineStr">
-        <is>
-          <t>If below 0.80: defer the next purchase order, review pack-size-driven over-ordering, and check that issues are recorded daily. If above 1.05: confirm the stock position and re-base the requisition quantity.</t>
-        </is>
-      </c>
-      <c r="I5" s="11" t="inlineStr">
-        <is>
-          <t>At month close, before the next requisition cycle.</t>
-        </is>
-      </c>
-      <c r="J5" s="11" t="inlineStr">
-        <is>
-          <t>Head of Procurement → Director Finance &amp; Operations</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="132" customHeight="1">
-      <c r="A6" s="10" t="inlineStr">
-        <is>
-          <t>CM-02</t>
-        </is>
-      </c>
-      <c r="B6" s="11" t="inlineStr">
-        <is>
-          <t>Budget utilisation – Medical Consumables (FY2025-26)</t>
-        </is>
-      </c>
-      <c r="C6" s="11" t="inlineStr">
-        <is>
-          <t>151.4%</t>
-        </is>
-      </c>
-      <c r="D6" s="20" t="inlineStr">
-        <is>
-          <t>Red</t>
-        </is>
-      </c>
-      <c r="E6" s="11" t="inlineStr">
-        <is>
-          <t>Medical Consumables consumption of PKR 34,812,356 exceeds the approved budget of PKR 22,997,000 by PKR 11,815,356 (51.4%).</t>
-        </is>
-      </c>
-      <c r="F6" s="11" t="inlineStr">
-        <is>
-          <t>Ranked causes to test: (1) price increase on a major item; (2) service volume higher than planned; (3) category budget under-estimated at planning; (4) mis-posting from another category; (5) wastage replacement purchases. Test price first, using the price-variance view (D-17).</t>
-        </is>
-      </c>
-      <c r="G6" s="11" t="inlineStr">
-        <is>
-          <t>An over-committed category can only be funded by taking budget from another line or by new money; left unresolved it becomes a donor-reporting exception in FY2025-26.</t>
-        </is>
-      </c>
-      <c r="H6" s="11" t="inlineStr">
-        <is>
-          <t>Record written commentary with the price/volume split; reallocate from an under-utilised category (see CM-03); tighten issue authorisation for the category; renegotiate the top two items by value.</t>
-        </is>
-      </c>
-      <c r="I6" s="11" t="inlineStr">
-        <is>
-          <t>Within 3 working days of the month close; reallocation before the fiscal year reaches 75% elapsed.</t>
-        </is>
-      </c>
-      <c r="J6" s="11" t="inlineStr">
-        <is>
-          <t>Manager Finance &amp; Grants → Director Finance &amp; Operations</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="132" customHeight="1">
-      <c r="A7" s="10" t="inlineStr">
-        <is>
-          <t>CM-03</t>
-        </is>
-      </c>
-      <c r="B7" s="11" t="inlineStr">
-        <is>
-          <t>Budget utilisation – Equipment (FY2026-27)</t>
-        </is>
-      </c>
-      <c r="C7" s="11" t="inlineStr">
-        <is>
-          <t>0.1%</t>
-        </is>
-      </c>
-      <c r="D7" s="20" t="inlineStr">
-        <is>
-          <t>Red</t>
-        </is>
-      </c>
-      <c r="E7" s="11" t="inlineStr">
-        <is>
-          <t>Equipment budget of PKR 5,808,000 has used only PKR 6,782 (0.1%).</t>
-        </is>
-      </c>
-      <c r="F7" s="11" t="inlineStr">
-        <is>
-          <t>Ranked causes to test: (1) capital items stuck in approval or quotation; (2) requirement overstated at planning; (3) items recorded as consumables rather than equipment; (4) procurement deferred to the last quarter.</t>
-        </is>
-      </c>
-      <c r="G7" s="11" t="inlineStr">
-        <is>
-          <t>Under-utilisation is read by donors as slow implementation; at project end it becomes unspent budget and, if equipment is genuinely needed, a service-capability gap.</t>
-        </is>
-      </c>
-      <c r="H7" s="11" t="inlineStr">
-        <is>
-          <t>Review the equipment pipeline item by item; approve or cancel pending requests; either accelerate justified purchases or formally reallocate the budget to medicines and consumables before year end.</t>
-        </is>
-      </c>
-      <c r="I7" s="11" t="inlineStr">
-        <is>
-          <t>This quarter — capital purchases need the full procurement cycle before the fiscal year ends.</t>
-        </is>
-      </c>
-      <c r="J7" s="11" t="inlineStr">
-        <is>
-          <t>Head of Procurement → Director Programme</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="132" customHeight="1">
-      <c r="A8" s="10" t="inlineStr">
-        <is>
-          <t>CM-04</t>
-        </is>
-      </c>
-      <c r="B8" s="11" t="inlineStr">
-        <is>
-          <t>Unattributed consumption</t>
-        </is>
-      </c>
-      <c r="C8" s="11" t="inlineStr">
-        <is>
-          <t>2.4%</t>
-        </is>
-      </c>
-      <c r="D8" s="20" t="inlineStr">
-        <is>
-          <t>Red</t>
-        </is>
-      </c>
-      <c r="E8" s="11" t="inlineStr">
-        <is>
-          <t>PKR 6,271,241 of consumption (468 issue lines, 2.4% of value) is charged to a generic cost centre rather than a project. Worst month: Jan-2025.</t>
-        </is>
-      </c>
-      <c r="F8" s="11" t="inlineStr">
-        <is>
-          <t>Ranked causes to test: (1) a default or generic project code used as a shortcut at issue; (2) users not trained on project coding; (3) new project not yet set up in the system; (4) system default overriding the correct code. Cross-tabulate by user, warehouse and service point to identify the pattern.</t>
-        </is>
-      </c>
-      <c r="G8" s="11" t="inlineStr">
-        <is>
-          <t>Project-level consumption, cost per beneficiary and budget utilisation are all understated for the projects that actually consumed the stock, and overstated nowhere — the numbers do not add up to the total.</t>
-        </is>
-      </c>
-      <c r="H8" s="11" t="inlineStr">
-        <is>
-          <t>Correct retroactively where the consuming project is evidenced; make the project field mandatory and validated in Oracle; retrain the top users identified; add this exception to the monthly review agenda.</t>
-        </is>
-      </c>
-      <c r="I8" s="11" t="inlineStr">
-        <is>
-          <t>Correction within the current month; system control change within the quarter.</t>
-        </is>
-      </c>
-      <c r="J8" s="11" t="inlineStr">
-        <is>
-          <t>Head of Procurement (with IT) → Director Finance &amp; Operations</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="132" customHeight="1">
-      <c r="A9" s="10" t="inlineStr">
-        <is>
-          <t>CM-05</t>
-        </is>
-      </c>
-      <c r="B9" s="11" t="inlineStr">
-        <is>
-          <t>Expired and near-expiry stock</t>
-        </is>
-      </c>
-      <c r="C9" s="11" t="inlineStr">
-        <is>
-          <t>PKR 783,764 expired; PKR 950,940 within 60 days</t>
-        </is>
-      </c>
-      <c r="D9" s="20" t="inlineStr">
-        <is>
-          <t>Red</t>
-        </is>
-      </c>
-      <c r="E9" s="11" t="inlineStr">
-        <is>
-          <t>PKR 783,764 of stock (1.9% of stock value) is already past expiry and not written off; a further PKR 950,940 expires within 60 days and PKR 636,720 within 90 days. Largest expired item: Hand Sanitiser 500 ml.</t>
-        </is>
-      </c>
-      <c r="F9" s="11" t="inlineStr">
-        <is>
-          <t>Ranked causes to test: (1) short-dated stock accepted at receipt or received as a donation; (2) over-ordering against an estimate rather than consumption; (3) stock held in the wrong warehouse or project; (4) protocol change making the item obsolete; (5) unrecorded consumption.</t>
-        </is>
-      </c>
-      <c r="G9" s="11" t="inlineStr">
-        <is>
-          <t>Direct, avoidable financial loss, plus a probable audit observation on stock management and donor reporting on commodity end-use.</t>
-        </is>
-      </c>
-      <c r="H9" s="11" t="inlineStr">
-        <is>
-          <t>Approve and record the write-off; redistribute the near-expiry balance to a project with demand; enforce first-expiry-first-out issue; reject short-dated deliveries at receipt; freeze ordering of the affected items.</t>
-        </is>
-      </c>
-      <c r="I9" s="11" t="inlineStr">
-        <is>
-          <t>Within 5 working days of the expiry flag; write-off before the financial year closes.</t>
-        </is>
-      </c>
-      <c r="J9" s="11" t="inlineStr">
-        <is>
-          <t>Stores in-charge → Head of Procurement</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="132" customHeight="1">
-      <c r="A10" s="10" t="inlineStr">
-        <is>
-          <t>CM-06</t>
-        </is>
-      </c>
-      <c r="B10" s="11" t="inlineStr">
-        <is>
-          <t>Stock cover / stock-out risk</t>
-        </is>
-      </c>
-      <c r="C10" s="11" t="inlineStr">
-        <is>
-          <t>3 items below 60 days; lowest 32 days (F-100 Therapeutic Milk 400 g)</t>
-        </is>
-      </c>
-      <c r="D10" s="21" t="inlineStr">
-        <is>
-          <t>Amber</t>
-        </is>
-      </c>
-      <c r="E10" s="11" t="inlineStr">
-        <is>
-          <t>0 items are below 30 days of cover and 3 below 60 days, against an average supplier lead time of 32 days.</t>
-        </is>
-      </c>
-      <c r="F10" s="11" t="inlineStr">
-        <is>
-          <t>Ranked causes to test: (1) lead time longer than the assumption used in planning; (2) demand surge above trend; (3) partial delivery or delayed GRN; (4) stock transferred out to another project; (5) pack size forcing under-supply.</t>
-        </is>
-      </c>
-      <c r="G10" s="11" t="inlineStr">
-        <is>
-          <t>A stock-out of a critical medicine interrupts service delivery and forces an emergency purchase at a higher price — the most expensive way to buy.</t>
-        </is>
-      </c>
-      <c r="H10" s="11" t="inlineStr">
-        <is>
-          <t>Raise a fast-track purchase for items where cover is below lead time; transfer stock from a warehouse with surplus cover; agree a temporary substitution with the clinical lead where clinically acceptable.</t>
-        </is>
-      </c>
-      <c r="I10" s="11" t="inlineStr">
-        <is>
-          <t>Immediately where cover is below lead time; same day for clinical items.</t>
-        </is>
-      </c>
-      <c r="J10" s="11" t="inlineStr">
-        <is>
-          <t>Stores in-charge (with Procurement) → Head of Procurement</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="132" customHeight="1">
-      <c r="A11" s="10" t="inlineStr">
-        <is>
-          <t>CM-07</t>
-        </is>
-      </c>
-      <c r="B11" s="11" t="inlineStr">
-        <is>
-          <t>Slow-moving and overstocked items</t>
-        </is>
-      </c>
-      <c r="C11" s="11" t="inlineStr">
-        <is>
-          <t>5 items, PKR 168,300; PKR 3,446,230 with over 180 days cover</t>
-        </is>
-      </c>
-      <c r="D11" s="21" t="inlineStr">
-        <is>
-          <t>Amber</t>
-        </is>
-      </c>
-      <c r="E11" s="11" t="inlineStr">
-        <is>
-          <t>5 items have no consumption in the last 90 days and PKR 3,446,230 of stock represents more than 180 days of cover. Stock on hand totals PKR 41,090,444.</t>
-        </is>
-      </c>
-      <c r="F11" s="11" t="inlineStr">
-        <is>
-          <t>Ranked causes to test: (1) demand over-estimated at requisition; (2) item superseded or removed from the protocol; (3) stock received for a project that has since reduced activity; (4) wrong warehouse allocation.</t>
-        </is>
-      </c>
-      <c r="G11" s="11" t="inlineStr">
-        <is>
-          <t>Blocked working capital and a future expiry loss; it also distorts the consumption-to-investment ratio.</t>
-        </is>
-      </c>
-      <c r="H11" s="11" t="inlineStr">
-        <is>
-          <t>Freeze re-ordering and set a review date; redistribute to a consuming project; correct the requirement formula with actual consumption; plan disposal or return for what cannot be consumed.</t>
-        </is>
-      </c>
-      <c r="I11" s="11" t="inlineStr">
-        <is>
-          <t>Freeze immediately; disposition before the expiry alert window.</t>
-        </is>
-      </c>
-      <c r="J11" s="11" t="inlineStr">
-        <is>
-          <t>Supply Chain Officer → Head of Procurement</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="132" customHeight="1">
-      <c r="A12" s="10" t="inlineStr">
-        <is>
-          <t>CM-08</t>
-        </is>
-      </c>
-      <c r="B12" s="11" t="inlineStr">
-        <is>
-          <t>Price variance</t>
-        </is>
-      </c>
-      <c r="C12" s="11" t="inlineStr">
-        <is>
-          <t>Average +16.2%; highest Diclofenac 75 mg Injection +19.4%</t>
-        </is>
-      </c>
-      <c r="D12" s="21" t="inlineStr">
-        <is>
-          <t>Amber</t>
-        </is>
-      </c>
-      <c r="E12" s="11" t="inlineStr">
-        <is>
-          <t>Across 77 items with comparable purchases, the weighted average unit price rose 16.2% between the first and latest purchase; Diclofenac 75 mg Injection rose from 28.99 to 34.63 (19.4%).</t>
-        </is>
-      </c>
-      <c r="F12" s="11" t="inlineStr">
-        <is>
-          <t>Ranked causes to test: (1) market or exchange-rate movement; (2) loss of contract price or supplier change; (3) specification or pack-size change; (4) emergency or split purchase at a higher price; (5) unit-of-measure error in the PO.</t>
-        </is>
-      </c>
-      <c r="G12" s="11" t="inlineStr">
-        <is>
-          <t>Price movement consumes budget without any change in service volume, so activity has to be reduced later in the year unless it is negotiated or re-budgeted.</t>
-        </is>
-      </c>
-      <c r="H12" s="11" t="inlineStr">
-        <is>
-          <t>Re-quote or invoke contract terms for the top five risers; consolidate demand to restore volume discounts; verify specification and UOM; record the price effect separately in the variance commentary.</t>
-        </is>
-      </c>
-      <c r="I12" s="11" t="inlineStr">
-        <is>
-          <t>Before the next contract or purchase cycle.</t>
-        </is>
-      </c>
-      <c r="J12" s="11" t="inlineStr">
-        <is>
-          <t>Procurement Officer → Head of Procurement</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="132" customHeight="1">
-      <c r="A13" s="10" t="inlineStr">
-        <is>
-          <t>CM-09</t>
-        </is>
-      </c>
-      <c r="B13" s="11" t="inlineStr">
-        <is>
-          <t>Open commitments and cancelled orders</t>
-        </is>
-      </c>
-      <c r="C13" s="11" t="inlineStr">
-        <is>
-          <t>PKR 4,467,951 open; 847 lines cancelled (PKR 18,943,642)</t>
-        </is>
-      </c>
-      <c r="D13" s="21" t="inlineStr">
-        <is>
-          <t>Amber</t>
-        </is>
-      </c>
-      <c r="E13" s="11" t="inlineStr">
-        <is>
-          <t>320 PO lines worth PKR 4,467,951 remain un-received, and 847 lines worth PKR 18,943,642 were cancelled in the period.</t>
-        </is>
-      </c>
-      <c r="F13" s="11" t="inlineStr">
-        <is>
-          <t>Ranked causes to test: (1) supplier capacity or import delay; (2) budget hold or approval delay; (3) requirement changed after ordering; (4) split ordering to stay within approval limits.</t>
-        </is>
-      </c>
-      <c r="G13" s="11" t="inlineStr">
-        <is>
-          <t>Open commitments are future cash outflows and future stock; cancellations indicate that requisitions were raised before the need was firm, which wastes procurement capacity.</t>
-        </is>
-      </c>
-      <c r="H13" s="11" t="inlineStr">
-        <is>
-          <t>Confirm delivery dates in writing; re-plan or cancel the balance where the need has changed; review approval thresholds if split ordering is evident; use the commitment figure in cash planning.</t>
-        </is>
-      </c>
-      <c r="I13" s="11" t="inlineStr">
-        <is>
-          <t>Weekly review; escalate any line open for more than 30 days.</t>
-        </is>
-      </c>
-      <c r="J13" s="11" t="inlineStr">
-        <is>
-          <t>Procurement Officer → Manager Finance</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="132" customHeight="1">
-      <c r="A14" s="10" t="inlineStr">
-        <is>
-          <t>CM-10</t>
-        </is>
-      </c>
-      <c r="B14" s="11" t="inlineStr">
-        <is>
-          <t>Projects ending soon with unspent budget</t>
-        </is>
-      </c>
-      <c r="C14" s="11" t="inlineStr">
-        <is>
-          <t>6 projects; PKR 136,478,187 unspent</t>
-        </is>
-      </c>
-      <c r="D14" s="20" t="inlineStr">
-        <is>
-          <t>Red</t>
-        </is>
-      </c>
-      <c r="E14" s="11" t="inlineStr">
-        <is>
-          <t>6 projects end within 120 days with a combined PKR 136,478,187 of budget unspent (largest: Maternal &amp; Child Health Programme - Kora, PKR 33,322,723).</t>
-        </is>
-      </c>
-      <c r="F14" s="11" t="inlineStr">
-        <is>
-          <t>Ranked causes to test: (1) activity slower than plan; (2) budget allocated but never requisitioned; (3) consumption recorded against another project; (4) procurement capacity constraint; (5) budget overstated at award.</t>
-        </is>
-      </c>
-      <c r="G14" s="11" t="inlineStr">
-        <is>
-          <t>Unspent budget at project end is reported to donors as under-delivery and may be recovered; correcting it at the last minute usually produces poor-quality spending.</t>
-        </is>
-      </c>
-      <c r="H14" s="11" t="inlineStr">
-        <is>
-          <t>Prepare an end-of-project plan now: accelerate committed activity, procure only justified items, request a no-cost extension where activity remains, or return the balance formally.</t>
-        </is>
-      </c>
-      <c r="I14" s="11" t="inlineStr">
-        <is>
-          <t>This month — the procurement cycle must still fit inside the remaining period.</t>
-        </is>
-      </c>
-      <c r="J14" s="11" t="inlineStr">
-        <is>
-          <t>Programme Manager (with Finance) → Director Programme</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="132" customHeight="1">
-      <c r="A15" s="10" t="inlineStr">
-        <is>
-          <t>CM-11</t>
-        </is>
-      </c>
-      <c r="B15" s="11" t="inlineStr">
-        <is>
-          <t>Projected FY2026-27 funding position</t>
-        </is>
-      </c>
-      <c r="C15" s="11" t="inlineStr">
-        <is>
-          <t>projected PKR 135,073,508 vs budget PKR 67,078,000; gap PKR 67,995,508</t>
-        </is>
-      </c>
-      <c r="D15" s="20" t="inlineStr">
-        <is>
-          <t>Red</t>
-        </is>
-      </c>
-      <c r="E15" s="11" t="inlineStr">
-        <is>
-          <t>With 3 months elapsed and PKR 33,768,377 consumed, the burn rate of PKR 11,256,126 per month projects PKR 135,073,508 for the full year against a product budget of PKR 67,078,000.</t>
-        </is>
-      </c>
-      <c r="F15" s="11" t="inlineStr">
-        <is>
-          <t>Ranked causes to test: (1) budget phasing not yet loaded for the year; (2) genuine under-budgeting against price inflation; (3) consumption running above the planned service volume; (4) prior-year carry-over spend landing in this year.</t>
-        </is>
-      </c>
-      <c r="G15" s="11" t="inlineStr">
-        <is>
-          <t>If the gap is real, service levels cannot be maintained for the full year and the shortfall appears unannounced in the last quarter.</t>
-        </is>
-      </c>
-      <c r="H15" s="11" t="inlineStr">
-        <is>
-          <t>Confirm budget phasing with Finance first; if the gap is real, quantify it by project and category, prioritise spending on critical items, and raise a funding request or reprioritise activity with the donor.</t>
-        </is>
-      </c>
-      <c r="I15" s="11" t="inlineStr">
-        <is>
-          <t>Now, at the first quarter of the fiscal year — not at the ninth month.</t>
-        </is>
-      </c>
-      <c r="J15" s="11" t="inlineStr">
-        <is>
-          <t>Manager Finance &amp; Grants → Director Finance &amp; Operations</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="132" customHeight="1">
-      <c r="A16" s="10" t="inlineStr">
-        <is>
-          <t>CM-12</t>
-        </is>
-      </c>
-      <c r="B16" s="11" t="inlineStr">
-        <is>
-          <t>Cost per beneficiary (peer comparison)</t>
-        </is>
-      </c>
-      <c r="C16" s="11" t="inlineStr">
-        <is>
-          <t>overall PKR 385; range Hepatitis B &amp; C Screening -  PKR 227 to Nutrition Stabilisation Cent PKR 500</t>
-        </is>
-      </c>
-      <c r="D16" s="21" t="inlineStr">
-        <is>
-          <t>Amber</t>
-        </is>
-      </c>
-      <c r="E16" s="11" t="inlineStr">
-        <is>
-          <t>Product cost per beneficiary is PKR 385 across the portfolio, but ranges from PKR 227 in Hepatitis B &amp; C Screening - Keamari to PKR 500 in Nutrition Stabilisation Centre - Malir (a spread of 120.8%).</t>
-        </is>
-      </c>
-      <c r="F16" s="11" t="inlineStr">
-        <is>
-          <t>Ranked causes to test: (1) case mix and acuity of the service; (2) price paid and supplier terms; (3) service volume below facility capacity; (4) wastage and expiry inflating cost; (5) one-off stock build in the period.</t>
-        </is>
-      </c>
-      <c r="G16" s="11" t="inlineStr">
-        <is>
-          <t>A high cost per beneficiary relative to peers is the first question a donor asks; without an explanation it is read as inefficiency.</t>
-        </is>
-      </c>
-      <c r="H16" s="11" t="inlineStr">
-        <is>
-          <t>Normalise for category mix before drawing conclusions; address the identified driver (price, volume or waste); set an efficiency target for the next quarter and report the measure with its methodology.</t>
-        </is>
-      </c>
-      <c r="I16" s="11" t="inlineStr">
-        <is>
-          <t>Quarterly review, with the methodology published alongside the first report.</t>
-        </is>
-      </c>
-      <c r="J16" s="11" t="inlineStr">
-        <is>
-          <t>Director Programme → Executive management</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="132" customHeight="1">
-      <c r="A17" s="10" t="inlineStr">
-        <is>
-          <t>CM-13</t>
-        </is>
-      </c>
-      <c r="B17" s="11" t="inlineStr">
-        <is>
-          <t>Seasonality and peak readiness</t>
-        </is>
-      </c>
-      <c r="C17" s="11" t="inlineStr">
-        <is>
-          <t>peak month Aug-2025 (PKR 14,731,533); seasonal index highest in Jan at 1.23</t>
-        </is>
-      </c>
-      <c r="D17" s="21" t="inlineStr">
-        <is>
-          <t>Amber</t>
-        </is>
-      </c>
-      <c r="E17" s="11" t="inlineStr">
-        <is>
-          <t>Consumption peaks in Aug-2025 at PKR 14,731,533, 52.1% above the period average; the seasonal index is highest in Jan (1.23×) and lowest in Mar (0.83×).</t>
-        </is>
-      </c>
-      <c r="F17" s="11" t="inlineStr">
-        <is>
-          <t>Seasonal demand is driven by disease pattern (diarrhoeal and vector-borne illness in the monsoon months), campaign activity and beneficiary inflow; the peak is structural, not a one-off.</t>
-        </is>
-      </c>
-      <c r="G17" s="11" t="inlineStr">
-        <is>
-          <t>If stock is purchased during the surge rather than before it, the peak is met with emergency purchases at higher prices and with stock-outs at the moment of greatest need.</t>
-        </is>
-      </c>
-      <c r="H17" s="11" t="inlineStr">
-        <is>
-          <t>Pre-position peak quantities at least one lead time before the peak month; align the purchase plan and warehouse capacity with the seasonal index; review the index each quarter.</t>
-        </is>
-      </c>
-      <c r="I17" s="11" t="inlineStr">
-        <is>
-          <t>Two months before the peak season, every year.</t>
-        </is>
-      </c>
-      <c r="J17" s="11" t="inlineStr">
-        <is>
-          <t>Supply Chain Officer → Head of Procurement</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="132" customHeight="1">
-      <c r="A18" s="10" t="inlineStr">
-        <is>
-          <t>CM-14</t>
-        </is>
-      </c>
-      <c r="B18" s="11" t="inlineStr">
-        <is>
-          <t>Data quality and load integrity</t>
-        </is>
-      </c>
-      <c r="C18" s="11" t="inlineStr">
-        <is>
-          <t>8 duplicate receipts; 59 zero-price lines; 2 inactive items; 1 blacklisted supplier</t>
-        </is>
-      </c>
-      <c r="D18" s="21" t="inlineStr">
-        <is>
-          <t>Amber</t>
-        </is>
-      </c>
-      <c r="E18" s="11" t="inlineStr">
-        <is>
-          <t>The load contains 8 duplicate receipt candidates, 59 purchase lines at zero value, 2 inactive items with transaction history and 1 blacklisted supplier still appearing in purchase orders.</t>
-        </is>
-      </c>
-      <c r="F18" s="11" t="inlineStr">
-        <is>
-          <t>Ranked causes to test: (1) double posting in the source system; (2) in-kind or donated stock genuinely at zero value; (3) master data not maintained after item or supplier deactivation; (4) extract mapping or UOM error.</t>
-        </is>
-      </c>
-      <c r="G18" s="11" t="inlineStr">
-        <is>
-          <t>Each defect flows into a reported KPI: duplicates inflate stock and receipts, zero prices distort average price, and inactive data hides real consumption.</t>
-        </is>
-      </c>
-      <c r="H18" s="11" t="inlineStr">
-        <is>
-          <t>Deduplicate and correct at source before the next refresh; exclude zero-value lines from price analysis and disclose them as in-kind; clean the master data; add the check to the load gate.</t>
-        </is>
-      </c>
-      <c r="I18" s="11" t="inlineStr">
-        <is>
-          <t>Before the next refresh; defects recurring for three periods require a process change.</t>
-        </is>
-      </c>
-      <c r="J18" s="11" t="inlineStr">
-        <is>
-          <t>IT / BI → Head of Procurement</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Rule: no commentary without a number, no number without a cause, no cause without an action, no action without an owner and a date.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A4:J18"/>
-  <mergeCells count="1">
-    <mergeCell ref="A2:J2"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>